<commit_message>
[feat] add Partial Fullfilled
</commit_message>
<xml_diff>
--- a/addons/it_asset/static/excel_templates/material_request_template.xlsx
+++ b/addons/it_asset/static/excel_templates/material_request_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\10.PROJECT\odoo\addons\it_asset\static\excel_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{587F0986-0AE2-42DD-A10B-8FFD4ADB4BA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A9DB57B-EA38-4900-BD43-BB3708363A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
   <si>
     <t>FORM / FORMULIR</t>
   </si>
@@ -124,10 +124,22 @@
     <t>Tanggal :</t>
   </si>
   <si>
-    <t>Diketahui Oleh</t>
+    <t>GSI4-SCM-001A</t>
   </si>
   <si>
-    <t>GSI4-SCM-001A</t>
+    <t>Diperiksa Oleh</t>
+  </si>
+  <si>
+    <t>Diverifikasi Oleh</t>
+  </si>
+  <si>
+    <t>Diketahui Oleh,</t>
+  </si>
+  <si>
+    <t>Supt. HRGA</t>
+  </si>
+  <si>
+    <t>IT Supervisor</t>
   </si>
 </sst>
 </file>
@@ -1008,182 +1020,32 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1245,6 +1107,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1266,35 +1134,179 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1649,217 +1661,217 @@
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
-      <c r="G1" s="34" t="s">
+      <c r="G1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-      <c r="X1" s="35"/>
-      <c r="Y1" s="35"/>
-      <c r="Z1" s="35"/>
-      <c r="AA1" s="35"/>
-      <c r="AB1" s="35"/>
-      <c r="AC1" s="35"/>
-      <c r="AD1" s="35"/>
-      <c r="AE1" s="35"/>
-      <c r="AF1" s="35"/>
-      <c r="AG1" s="35"/>
-      <c r="AH1" s="35"/>
-      <c r="AI1" s="35"/>
-      <c r="AJ1" s="35"/>
-      <c r="AK1" s="35"/>
-      <c r="AL1" s="35"/>
-      <c r="AM1" s="35"/>
-      <c r="AN1" s="35"/>
-      <c r="AO1" s="35"/>
-      <c r="AP1" s="35"/>
-      <c r="AQ1" s="35"/>
-      <c r="AR1" s="35"/>
-      <c r="AS1" s="35"/>
-      <c r="AT1" s="35"/>
-      <c r="AU1" s="35"/>
-      <c r="AV1" s="35"/>
-      <c r="AW1" s="35"/>
-      <c r="AX1" s="35"/>
-      <c r="AY1" s="35"/>
-      <c r="AZ1" s="36"/>
-      <c r="BA1" s="37" t="s">
+      <c r="H1" s="105"/>
+      <c r="I1" s="105"/>
+      <c r="J1" s="105"/>
+      <c r="K1" s="105"/>
+      <c r="L1" s="105"/>
+      <c r="M1" s="105"/>
+      <c r="N1" s="105"/>
+      <c r="O1" s="105"/>
+      <c r="P1" s="105"/>
+      <c r="Q1" s="105"/>
+      <c r="R1" s="105"/>
+      <c r="S1" s="105"/>
+      <c r="T1" s="105"/>
+      <c r="U1" s="105"/>
+      <c r="V1" s="105"/>
+      <c r="W1" s="105"/>
+      <c r="X1" s="105"/>
+      <c r="Y1" s="105"/>
+      <c r="Z1" s="105"/>
+      <c r="AA1" s="105"/>
+      <c r="AB1" s="105"/>
+      <c r="AC1" s="105"/>
+      <c r="AD1" s="105"/>
+      <c r="AE1" s="105"/>
+      <c r="AF1" s="105"/>
+      <c r="AG1" s="105"/>
+      <c r="AH1" s="105"/>
+      <c r="AI1" s="105"/>
+      <c r="AJ1" s="105"/>
+      <c r="AK1" s="105"/>
+      <c r="AL1" s="105"/>
+      <c r="AM1" s="105"/>
+      <c r="AN1" s="105"/>
+      <c r="AO1" s="105"/>
+      <c r="AP1" s="105"/>
+      <c r="AQ1" s="105"/>
+      <c r="AR1" s="105"/>
+      <c r="AS1" s="105"/>
+      <c r="AT1" s="105"/>
+      <c r="AU1" s="105"/>
+      <c r="AV1" s="105"/>
+      <c r="AW1" s="105"/>
+      <c r="AX1" s="105"/>
+      <c r="AY1" s="105"/>
+      <c r="AZ1" s="106"/>
+      <c r="BA1" s="107" t="s">
         <v>1</v>
       </c>
-      <c r="BB1" s="38"/>
-      <c r="BC1" s="38"/>
-      <c r="BD1" s="38"/>
-      <c r="BE1" s="38"/>
-      <c r="BF1" s="39"/>
+      <c r="BB1" s="108"/>
+      <c r="BC1" s="108"/>
+      <c r="BD1" s="108"/>
+      <c r="BE1" s="108"/>
+      <c r="BF1" s="109"/>
       <c r="BG1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="BH1" s="38" t="s">
-        <v>30</v>
+      <c r="BH1" s="108" t="s">
+        <v>29</v>
       </c>
-      <c r="BI1" s="38"/>
-      <c r="BJ1" s="38"/>
-      <c r="BK1" s="38"/>
-      <c r="BL1" s="38"/>
-      <c r="BM1" s="39"/>
+      <c r="BI1" s="108"/>
+      <c r="BJ1" s="108"/>
+      <c r="BK1" s="108"/>
+      <c r="BL1" s="108"/>
+      <c r="BM1" s="109"/>
     </row>
     <row r="2" spans="2:65" ht="14.25" customHeight="1">
       <c r="B2" s="5"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="35"/>
-      <c r="P2" s="35"/>
-      <c r="Q2" s="35"/>
-      <c r="R2" s="35"/>
-      <c r="S2" s="35"/>
-      <c r="T2" s="35"/>
-      <c r="U2" s="35"/>
-      <c r="V2" s="35"/>
-      <c r="W2" s="35"/>
-      <c r="X2" s="35"/>
-      <c r="Y2" s="35"/>
-      <c r="Z2" s="35"/>
-      <c r="AA2" s="35"/>
-      <c r="AB2" s="35"/>
-      <c r="AC2" s="35"/>
-      <c r="AD2" s="35"/>
-      <c r="AE2" s="35"/>
-      <c r="AF2" s="35"/>
-      <c r="AG2" s="35"/>
-      <c r="AH2" s="35"/>
-      <c r="AI2" s="35"/>
-      <c r="AJ2" s="35"/>
-      <c r="AK2" s="35"/>
-      <c r="AL2" s="35"/>
-      <c r="AM2" s="35"/>
-      <c r="AN2" s="35"/>
-      <c r="AO2" s="35"/>
-      <c r="AP2" s="35"/>
-      <c r="AQ2" s="35"/>
-      <c r="AR2" s="35"/>
-      <c r="AS2" s="35"/>
-      <c r="AT2" s="35"/>
-      <c r="AU2" s="35"/>
-      <c r="AV2" s="35"/>
-      <c r="AW2" s="35"/>
-      <c r="AX2" s="35"/>
-      <c r="AY2" s="35"/>
-      <c r="AZ2" s="36"/>
-      <c r="BA2" s="40" t="s">
+      <c r="G2" s="104"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="105"/>
+      <c r="L2" s="105"/>
+      <c r="M2" s="105"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="105"/>
+      <c r="P2" s="105"/>
+      <c r="Q2" s="105"/>
+      <c r="R2" s="105"/>
+      <c r="S2" s="105"/>
+      <c r="T2" s="105"/>
+      <c r="U2" s="105"/>
+      <c r="V2" s="105"/>
+      <c r="W2" s="105"/>
+      <c r="X2" s="105"/>
+      <c r="Y2" s="105"/>
+      <c r="Z2" s="105"/>
+      <c r="AA2" s="105"/>
+      <c r="AB2" s="105"/>
+      <c r="AC2" s="105"/>
+      <c r="AD2" s="105"/>
+      <c r="AE2" s="105"/>
+      <c r="AF2" s="105"/>
+      <c r="AG2" s="105"/>
+      <c r="AH2" s="105"/>
+      <c r="AI2" s="105"/>
+      <c r="AJ2" s="105"/>
+      <c r="AK2" s="105"/>
+      <c r="AL2" s="105"/>
+      <c r="AM2" s="105"/>
+      <c r="AN2" s="105"/>
+      <c r="AO2" s="105"/>
+      <c r="AP2" s="105"/>
+      <c r="AQ2" s="105"/>
+      <c r="AR2" s="105"/>
+      <c r="AS2" s="105"/>
+      <c r="AT2" s="105"/>
+      <c r="AU2" s="105"/>
+      <c r="AV2" s="105"/>
+      <c r="AW2" s="105"/>
+      <c r="AX2" s="105"/>
+      <c r="AY2" s="105"/>
+      <c r="AZ2" s="106"/>
+      <c r="BA2" s="110" t="s">
         <v>3</v>
       </c>
-      <c r="BB2" s="41"/>
-      <c r="BC2" s="41"/>
-      <c r="BD2" s="41"/>
-      <c r="BE2" s="41"/>
-      <c r="BF2" s="42"/>
+      <c r="BB2" s="111"/>
+      <c r="BC2" s="111"/>
+      <c r="BD2" s="111"/>
+      <c r="BE2" s="111"/>
+      <c r="BF2" s="112"/>
       <c r="BG2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="BH2" s="41">
+      <c r="BH2" s="111">
         <v>1</v>
       </c>
-      <c r="BI2" s="41"/>
-      <c r="BJ2" s="41"/>
-      <c r="BK2" s="41"/>
-      <c r="BL2" s="41"/>
-      <c r="BM2" s="42"/>
+      <c r="BI2" s="111"/>
+      <c r="BJ2" s="111"/>
+      <c r="BK2" s="111"/>
+      <c r="BL2" s="111"/>
+      <c r="BM2" s="112"/>
     </row>
     <row r="3" spans="2:65" ht="14.25" customHeight="1">
       <c r="B3" s="5"/>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="44" t="s">
+      <c r="G3" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
-      <c r="N3" s="45"/>
-      <c r="O3" s="45"/>
-      <c r="P3" s="45"/>
-      <c r="Q3" s="45"/>
-      <c r="R3" s="45"/>
-      <c r="S3" s="45"/>
-      <c r="T3" s="45"/>
-      <c r="U3" s="45"/>
-      <c r="V3" s="45"/>
-      <c r="W3" s="45"/>
-      <c r="X3" s="45"/>
-      <c r="Y3" s="45"/>
-      <c r="Z3" s="45"/>
-      <c r="AA3" s="45"/>
-      <c r="AB3" s="45"/>
-      <c r="AC3" s="45"/>
-      <c r="AD3" s="45"/>
-      <c r="AE3" s="45"/>
-      <c r="AF3" s="45"/>
-      <c r="AG3" s="45"/>
-      <c r="AH3" s="45"/>
-      <c r="AI3" s="45"/>
-      <c r="AJ3" s="45"/>
-      <c r="AK3" s="45"/>
-      <c r="AL3" s="45"/>
-      <c r="AM3" s="45"/>
-      <c r="AN3" s="45"/>
-      <c r="AO3" s="45"/>
-      <c r="AP3" s="45"/>
-      <c r="AQ3" s="45"/>
-      <c r="AR3" s="45"/>
-      <c r="AS3" s="45"/>
-      <c r="AT3" s="45"/>
-      <c r="AU3" s="45"/>
-      <c r="AV3" s="45"/>
-      <c r="AW3" s="45"/>
-      <c r="AX3" s="45"/>
-      <c r="AY3" s="45"/>
-      <c r="AZ3" s="46"/>
-      <c r="BA3" s="47" t="s">
+      <c r="H3" s="114"/>
+      <c r="I3" s="114"/>
+      <c r="J3" s="114"/>
+      <c r="K3" s="114"/>
+      <c r="L3" s="114"/>
+      <c r="M3" s="114"/>
+      <c r="N3" s="114"/>
+      <c r="O3" s="114"/>
+      <c r="P3" s="114"/>
+      <c r="Q3" s="114"/>
+      <c r="R3" s="114"/>
+      <c r="S3" s="114"/>
+      <c r="T3" s="114"/>
+      <c r="U3" s="114"/>
+      <c r="V3" s="114"/>
+      <c r="W3" s="114"/>
+      <c r="X3" s="114"/>
+      <c r="Y3" s="114"/>
+      <c r="Z3" s="114"/>
+      <c r="AA3" s="114"/>
+      <c r="AB3" s="114"/>
+      <c r="AC3" s="114"/>
+      <c r="AD3" s="114"/>
+      <c r="AE3" s="114"/>
+      <c r="AF3" s="114"/>
+      <c r="AG3" s="114"/>
+      <c r="AH3" s="114"/>
+      <c r="AI3" s="114"/>
+      <c r="AJ3" s="114"/>
+      <c r="AK3" s="114"/>
+      <c r="AL3" s="114"/>
+      <c r="AM3" s="114"/>
+      <c r="AN3" s="114"/>
+      <c r="AO3" s="114"/>
+      <c r="AP3" s="114"/>
+      <c r="AQ3" s="114"/>
+      <c r="AR3" s="114"/>
+      <c r="AS3" s="114"/>
+      <c r="AT3" s="114"/>
+      <c r="AU3" s="114"/>
+      <c r="AV3" s="114"/>
+      <c r="AW3" s="114"/>
+      <c r="AX3" s="114"/>
+      <c r="AY3" s="114"/>
+      <c r="AZ3" s="115"/>
+      <c r="BA3" s="116" t="s">
         <v>5</v>
       </c>
-      <c r="BB3" s="48"/>
-      <c r="BC3" s="48"/>
-      <c r="BD3" s="48"/>
-      <c r="BE3" s="48"/>
-      <c r="BF3" s="49"/>
+      <c r="BB3" s="117"/>
+      <c r="BC3" s="117"/>
+      <c r="BD3" s="117"/>
+      <c r="BE3" s="117"/>
+      <c r="BF3" s="118"/>
       <c r="BG3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="BH3" s="43">
+      <c r="BH3" s="119">
         <v>45611</v>
       </c>
-      <c r="BI3" s="41"/>
-      <c r="BJ3" s="41"/>
-      <c r="BK3" s="41"/>
-      <c r="BL3" s="41"/>
-      <c r="BM3" s="42"/>
+      <c r="BI3" s="111"/>
+      <c r="BJ3" s="111"/>
+      <c r="BK3" s="111"/>
+      <c r="BL3" s="111"/>
+      <c r="BM3" s="112"/>
     </row>
     <row r="4" spans="2:65" ht="14.25" customHeight="1">
       <c r="B4" s="7"/>
@@ -1867,923 +1879,923 @@
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="45"/>
-      <c r="I4" s="45"/>
-      <c r="J4" s="45"/>
-      <c r="K4" s="45"/>
-      <c r="L4" s="45"/>
-      <c r="M4" s="45"/>
-      <c r="N4" s="45"/>
-      <c r="O4" s="45"/>
-      <c r="P4" s="45"/>
-      <c r="Q4" s="45"/>
-      <c r="R4" s="45"/>
-      <c r="S4" s="45"/>
-      <c r="T4" s="45"/>
-      <c r="U4" s="45"/>
-      <c r="V4" s="45"/>
-      <c r="W4" s="45"/>
-      <c r="X4" s="45"/>
-      <c r="Y4" s="45"/>
-      <c r="Z4" s="45"/>
-      <c r="AA4" s="45"/>
-      <c r="AB4" s="45"/>
-      <c r="AC4" s="45"/>
-      <c r="AD4" s="45"/>
-      <c r="AE4" s="45"/>
-      <c r="AF4" s="45"/>
-      <c r="AG4" s="45"/>
-      <c r="AH4" s="45"/>
-      <c r="AI4" s="45"/>
-      <c r="AJ4" s="45"/>
-      <c r="AK4" s="45"/>
-      <c r="AL4" s="45"/>
-      <c r="AM4" s="45"/>
-      <c r="AN4" s="45"/>
-      <c r="AO4" s="45"/>
-      <c r="AP4" s="45"/>
-      <c r="AQ4" s="45"/>
-      <c r="AR4" s="45"/>
-      <c r="AS4" s="45"/>
-      <c r="AT4" s="45"/>
-      <c r="AU4" s="45"/>
-      <c r="AV4" s="45"/>
-      <c r="AW4" s="45"/>
-      <c r="AX4" s="45"/>
-      <c r="AY4" s="45"/>
-      <c r="AZ4" s="46"/>
-      <c r="BA4" s="50" t="s">
+      <c r="G4" s="113"/>
+      <c r="H4" s="114"/>
+      <c r="I4" s="114"/>
+      <c r="J4" s="114"/>
+      <c r="K4" s="114"/>
+      <c r="L4" s="114"/>
+      <c r="M4" s="114"/>
+      <c r="N4" s="114"/>
+      <c r="O4" s="114"/>
+      <c r="P4" s="114"/>
+      <c r="Q4" s="114"/>
+      <c r="R4" s="114"/>
+      <c r="S4" s="114"/>
+      <c r="T4" s="114"/>
+      <c r="U4" s="114"/>
+      <c r="V4" s="114"/>
+      <c r="W4" s="114"/>
+      <c r="X4" s="114"/>
+      <c r="Y4" s="114"/>
+      <c r="Z4" s="114"/>
+      <c r="AA4" s="114"/>
+      <c r="AB4" s="114"/>
+      <c r="AC4" s="114"/>
+      <c r="AD4" s="114"/>
+      <c r="AE4" s="114"/>
+      <c r="AF4" s="114"/>
+      <c r="AG4" s="114"/>
+      <c r="AH4" s="114"/>
+      <c r="AI4" s="114"/>
+      <c r="AJ4" s="114"/>
+      <c r="AK4" s="114"/>
+      <c r="AL4" s="114"/>
+      <c r="AM4" s="114"/>
+      <c r="AN4" s="114"/>
+      <c r="AO4" s="114"/>
+      <c r="AP4" s="114"/>
+      <c r="AQ4" s="114"/>
+      <c r="AR4" s="114"/>
+      <c r="AS4" s="114"/>
+      <c r="AT4" s="114"/>
+      <c r="AU4" s="114"/>
+      <c r="AV4" s="114"/>
+      <c r="AW4" s="114"/>
+      <c r="AX4" s="114"/>
+      <c r="AY4" s="114"/>
+      <c r="AZ4" s="115"/>
+      <c r="BA4" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="BB4" s="51"/>
-      <c r="BC4" s="51"/>
-      <c r="BD4" s="51"/>
-      <c r="BE4" s="51"/>
-      <c r="BF4" s="52"/>
+      <c r="BB4" s="121"/>
+      <c r="BC4" s="121"/>
+      <c r="BD4" s="121"/>
+      <c r="BE4" s="121"/>
+      <c r="BF4" s="122"/>
       <c r="BG4" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="BH4" s="51">
+      <c r="BH4" s="121">
         <v>1</v>
       </c>
-      <c r="BI4" s="51"/>
-      <c r="BJ4" s="51"/>
-      <c r="BK4" s="51"/>
-      <c r="BL4" s="51"/>
-      <c r="BM4" s="52"/>
+      <c r="BI4" s="121"/>
+      <c r="BJ4" s="121"/>
+      <c r="BK4" s="121"/>
+      <c r="BL4" s="121"/>
+      <c r="BM4" s="122"/>
     </row>
     <row r="6" spans="2:65" ht="22.5" customHeight="1" thickTop="1">
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="97" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
+      <c r="C6" s="98"/>
+      <c r="D6" s="98"/>
+      <c r="E6" s="98"/>
+      <c r="F6" s="98"/>
+      <c r="G6" s="98"/>
       <c r="H6" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="I6" s="28"/>
-      <c r="J6" s="28"/>
-      <c r="K6" s="28"/>
-      <c r="L6" s="28"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28"/>
-      <c r="O6" s="28"/>
-      <c r="P6" s="28"/>
-      <c r="Q6" s="28"/>
-      <c r="R6" s="28"/>
-      <c r="S6" s="28"/>
-      <c r="T6" s="28"/>
-      <c r="U6" s="28"/>
-      <c r="V6" s="28"/>
-      <c r="W6" s="28"/>
-      <c r="X6" s="28"/>
-      <c r="Y6" s="28"/>
-      <c r="Z6" s="28"/>
-      <c r="AA6" s="28"/>
-      <c r="AB6" s="28"/>
-      <c r="AC6" s="28"/>
-      <c r="AD6" s="28"/>
-      <c r="AE6" s="28"/>
-      <c r="AF6" s="28"/>
-      <c r="AG6" s="28"/>
-      <c r="AH6" s="28"/>
-      <c r="AI6" s="28"/>
-      <c r="AJ6" s="28"/>
-      <c r="AK6" s="28"/>
-      <c r="AL6" s="28"/>
-      <c r="AM6" s="28"/>
-      <c r="AN6" s="28" t="s">
+      <c r="I6" s="98"/>
+      <c r="J6" s="98"/>
+      <c r="K6" s="98"/>
+      <c r="L6" s="98"/>
+      <c r="M6" s="98"/>
+      <c r="N6" s="98"/>
+      <c r="O6" s="98"/>
+      <c r="P6" s="98"/>
+      <c r="Q6" s="98"/>
+      <c r="R6" s="98"/>
+      <c r="S6" s="98"/>
+      <c r="T6" s="98"/>
+      <c r="U6" s="98"/>
+      <c r="V6" s="98"/>
+      <c r="W6" s="98"/>
+      <c r="X6" s="98"/>
+      <c r="Y6" s="98"/>
+      <c r="Z6" s="98"/>
+      <c r="AA6" s="98"/>
+      <c r="AB6" s="98"/>
+      <c r="AC6" s="98"/>
+      <c r="AD6" s="98"/>
+      <c r="AE6" s="98"/>
+      <c r="AF6" s="98"/>
+      <c r="AG6" s="98"/>
+      <c r="AH6" s="98"/>
+      <c r="AI6" s="98"/>
+      <c r="AJ6" s="98"/>
+      <c r="AK6" s="98"/>
+      <c r="AL6" s="98"/>
+      <c r="AM6" s="98"/>
+      <c r="AN6" s="98" t="s">
         <v>8</v>
       </c>
-      <c r="AO6" s="28"/>
-      <c r="AP6" s="28"/>
-      <c r="AQ6" s="28"/>
+      <c r="AO6" s="98"/>
+      <c r="AP6" s="98"/>
+      <c r="AQ6" s="98"/>
       <c r="AR6" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="AS6" s="28"/>
-      <c r="AT6" s="28"/>
-      <c r="AU6" s="28"/>
-      <c r="AV6" s="28"/>
-      <c r="AW6" s="28"/>
-      <c r="AX6" s="28"/>
-      <c r="AY6" s="28"/>
-      <c r="AZ6" s="28"/>
-      <c r="BA6" s="28"/>
-      <c r="BB6" s="28"/>
-      <c r="BC6" s="28"/>
-      <c r="BD6" s="28"/>
-      <c r="BE6" s="28"/>
-      <c r="BF6" s="28"/>
-      <c r="BG6" s="28"/>
-      <c r="BH6" s="28"/>
-      <c r="BI6" s="28"/>
-      <c r="BJ6" s="28"/>
-      <c r="BK6" s="28"/>
-      <c r="BL6" s="28"/>
-      <c r="BM6" s="29"/>
+      <c r="AS6" s="98"/>
+      <c r="AT6" s="98"/>
+      <c r="AU6" s="98"/>
+      <c r="AV6" s="98"/>
+      <c r="AW6" s="98"/>
+      <c r="AX6" s="98"/>
+      <c r="AY6" s="98"/>
+      <c r="AZ6" s="98"/>
+      <c r="BA6" s="98"/>
+      <c r="BB6" s="98"/>
+      <c r="BC6" s="98"/>
+      <c r="BD6" s="98"/>
+      <c r="BE6" s="98"/>
+      <c r="BF6" s="98"/>
+      <c r="BG6" s="98"/>
+      <c r="BH6" s="98"/>
+      <c r="BI6" s="98"/>
+      <c r="BJ6" s="98"/>
+      <c r="BK6" s="98"/>
+      <c r="BL6" s="98"/>
+      <c r="BM6" s="99"/>
     </row>
     <row r="7" spans="2:65" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="100" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="31"/>
+      <c r="C7" s="101"/>
+      <c r="D7" s="101"/>
+      <c r="E7" s="101"/>
+      <c r="F7" s="101"/>
+      <c r="G7" s="101"/>
       <c r="H7" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="I7" s="31" t="s">
+      <c r="I7" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="J7" s="31"/>
-      <c r="K7" s="31"/>
-      <c r="L7" s="31"/>
-      <c r="M7" s="31"/>
-      <c r="N7" s="31"/>
-      <c r="O7" s="31"/>
-      <c r="P7" s="31"/>
-      <c r="Q7" s="31"/>
-      <c r="R7" s="31"/>
-      <c r="S7" s="31"/>
-      <c r="T7" s="31"/>
-      <c r="U7" s="31"/>
-      <c r="V7" s="31"/>
-      <c r="W7" s="31"/>
-      <c r="X7" s="31"/>
-      <c r="Y7" s="31"/>
-      <c r="Z7" s="31"/>
-      <c r="AA7" s="31"/>
-      <c r="AB7" s="31"/>
-      <c r="AC7" s="31"/>
-      <c r="AD7" s="31"/>
-      <c r="AE7" s="31"/>
-      <c r="AF7" s="31"/>
-      <c r="AG7" s="31"/>
-      <c r="AH7" s="31"/>
-      <c r="AI7" s="31"/>
-      <c r="AJ7" s="31"/>
-      <c r="AK7" s="31"/>
-      <c r="AL7" s="31"/>
-      <c r="AM7" s="31"/>
-      <c r="AN7" s="31" t="s">
+      <c r="J7" s="101"/>
+      <c r="K7" s="101"/>
+      <c r="L7" s="101"/>
+      <c r="M7" s="101"/>
+      <c r="N7" s="101"/>
+      <c r="O7" s="101"/>
+      <c r="P7" s="101"/>
+      <c r="Q7" s="101"/>
+      <c r="R7" s="101"/>
+      <c r="S7" s="101"/>
+      <c r="T7" s="101"/>
+      <c r="U7" s="101"/>
+      <c r="V7" s="101"/>
+      <c r="W7" s="101"/>
+      <c r="X7" s="101"/>
+      <c r="Y7" s="101"/>
+      <c r="Z7" s="101"/>
+      <c r="AA7" s="101"/>
+      <c r="AB7" s="101"/>
+      <c r="AC7" s="101"/>
+      <c r="AD7" s="101"/>
+      <c r="AE7" s="101"/>
+      <c r="AF7" s="101"/>
+      <c r="AG7" s="101"/>
+      <c r="AH7" s="101"/>
+      <c r="AI7" s="101"/>
+      <c r="AJ7" s="101"/>
+      <c r="AK7" s="101"/>
+      <c r="AL7" s="101"/>
+      <c r="AM7" s="101"/>
+      <c r="AN7" s="101" t="s">
         <v>11</v>
       </c>
-      <c r="AO7" s="31"/>
-      <c r="AP7" s="31"/>
-      <c r="AQ7" s="31"/>
+      <c r="AO7" s="101"/>
+      <c r="AP7" s="101"/>
+      <c r="AQ7" s="101"/>
       <c r="AR7" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="AS7" s="32"/>
-      <c r="AT7" s="31"/>
-      <c r="AU7" s="31"/>
-      <c r="AV7" s="31"/>
-      <c r="AW7" s="31"/>
-      <c r="AX7" s="31"/>
-      <c r="AY7" s="31"/>
-      <c r="AZ7" s="31"/>
-      <c r="BA7" s="31"/>
-      <c r="BB7" s="31"/>
-      <c r="BC7" s="31"/>
-      <c r="BD7" s="31"/>
-      <c r="BE7" s="31"/>
-      <c r="BF7" s="31"/>
-      <c r="BG7" s="31"/>
-      <c r="BH7" s="31"/>
-      <c r="BI7" s="31"/>
-      <c r="BJ7" s="31"/>
-      <c r="BK7" s="31"/>
-      <c r="BL7" s="31"/>
-      <c r="BM7" s="33"/>
+      <c r="AS7" s="102"/>
+      <c r="AT7" s="101"/>
+      <c r="AU7" s="101"/>
+      <c r="AV7" s="101"/>
+      <c r="AW7" s="101"/>
+      <c r="AX7" s="101"/>
+      <c r="AY7" s="101"/>
+      <c r="AZ7" s="101"/>
+      <c r="BA7" s="101"/>
+      <c r="BB7" s="101"/>
+      <c r="BC7" s="101"/>
+      <c r="BD7" s="101"/>
+      <c r="BE7" s="101"/>
+      <c r="BF7" s="101"/>
+      <c r="BG7" s="101"/>
+      <c r="BH7" s="101"/>
+      <c r="BI7" s="101"/>
+      <c r="BJ7" s="101"/>
+      <c r="BK7" s="101"/>
+      <c r="BL7" s="101"/>
+      <c r="BM7" s="103"/>
     </row>
     <row r="8" spans="2:65" ht="15.75" thickTop="1" thickBot="1"/>
     <row r="9" spans="2:65" ht="19.5" customHeight="1" thickTop="1">
-      <c r="B9" s="68" t="s">
+      <c r="B9" s="88" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="55"/>
-      <c r="D9" s="70" t="s">
+      <c r="C9" s="79"/>
+      <c r="D9" s="90" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="71"/>
-      <c r="F9" s="71"/>
-      <c r="G9" s="71"/>
-      <c r="H9" s="72"/>
-      <c r="I9" s="70" t="s">
+      <c r="E9" s="91"/>
+      <c r="F9" s="91"/>
+      <c r="G9" s="91"/>
+      <c r="H9" s="92"/>
+      <c r="I9" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="J9" s="71"/>
-      <c r="K9" s="71"/>
-      <c r="L9" s="71"/>
-      <c r="M9" s="71"/>
-      <c r="N9" s="71"/>
-      <c r="O9" s="71"/>
-      <c r="P9" s="71"/>
-      <c r="Q9" s="71"/>
-      <c r="R9" s="71"/>
-      <c r="S9" s="71"/>
-      <c r="T9" s="71"/>
-      <c r="U9" s="72"/>
-      <c r="V9" s="53" t="s">
+      <c r="J9" s="91"/>
+      <c r="K9" s="91"/>
+      <c r="L9" s="91"/>
+      <c r="M9" s="91"/>
+      <c r="N9" s="91"/>
+      <c r="O9" s="91"/>
+      <c r="P9" s="91"/>
+      <c r="Q9" s="91"/>
+      <c r="R9" s="91"/>
+      <c r="S9" s="91"/>
+      <c r="T9" s="91"/>
+      <c r="U9" s="92"/>
+      <c r="V9" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="W9" s="53"/>
-      <c r="X9" s="53"/>
-      <c r="Y9" s="53"/>
-      <c r="Z9" s="53"/>
-      <c r="AA9" s="53"/>
-      <c r="AB9" s="53"/>
-      <c r="AC9" s="53"/>
-      <c r="AD9" s="53"/>
-      <c r="AE9" s="53"/>
-      <c r="AF9" s="53"/>
-      <c r="AG9" s="53"/>
-      <c r="AH9" s="53" t="s">
+      <c r="W9" s="77"/>
+      <c r="X9" s="77"/>
+      <c r="Y9" s="77"/>
+      <c r="Z9" s="77"/>
+      <c r="AA9" s="77"/>
+      <c r="AB9" s="77"/>
+      <c r="AC9" s="77"/>
+      <c r="AD9" s="77"/>
+      <c r="AE9" s="77"/>
+      <c r="AF9" s="77"/>
+      <c r="AG9" s="77"/>
+      <c r="AH9" s="77" t="s">
         <v>16</v>
       </c>
-      <c r="AI9" s="53"/>
-      <c r="AJ9" s="53"/>
-      <c r="AK9" s="53" t="s">
+      <c r="AI9" s="77"/>
+      <c r="AJ9" s="77"/>
+      <c r="AK9" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="AL9" s="53"/>
-      <c r="AM9" s="53"/>
-      <c r="AN9" s="53" t="s">
+      <c r="AL9" s="77"/>
+      <c r="AM9" s="77"/>
+      <c r="AN9" s="77" t="s">
         <v>18</v>
       </c>
-      <c r="AO9" s="53"/>
-      <c r="AP9" s="53"/>
-      <c r="AQ9" s="53"/>
-      <c r="AR9" s="53"/>
-      <c r="AS9" s="53"/>
-      <c r="AT9" s="53"/>
-      <c r="AU9" s="53" t="s">
+      <c r="AO9" s="77"/>
+      <c r="AP9" s="77"/>
+      <c r="AQ9" s="77"/>
+      <c r="AR9" s="77"/>
+      <c r="AS9" s="77"/>
+      <c r="AT9" s="77"/>
+      <c r="AU9" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="AV9" s="53"/>
-      <c r="AW9" s="53"/>
-      <c r="AX9" s="53"/>
-      <c r="AY9" s="53"/>
-      <c r="AZ9" s="53"/>
-      <c r="BA9" s="53"/>
-      <c r="BB9" s="53"/>
-      <c r="BC9" s="55" t="s">
+      <c r="AV9" s="77"/>
+      <c r="AW9" s="77"/>
+      <c r="AX9" s="77"/>
+      <c r="AY9" s="77"/>
+      <c r="AZ9" s="77"/>
+      <c r="BA9" s="77"/>
+      <c r="BB9" s="77"/>
+      <c r="BC9" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="BD9" s="55"/>
-      <c r="BE9" s="55"/>
-      <c r="BF9" s="55"/>
-      <c r="BG9" s="55"/>
-      <c r="BH9" s="55"/>
-      <c r="BI9" s="55"/>
-      <c r="BJ9" s="55"/>
-      <c r="BK9" s="55"/>
-      <c r="BL9" s="55"/>
-      <c r="BM9" s="56"/>
+      <c r="BD9" s="79"/>
+      <c r="BE9" s="79"/>
+      <c r="BF9" s="79"/>
+      <c r="BG9" s="79"/>
+      <c r="BH9" s="79"/>
+      <c r="BI9" s="79"/>
+      <c r="BJ9" s="79"/>
+      <c r="BK9" s="79"/>
+      <c r="BL9" s="79"/>
+      <c r="BM9" s="80"/>
     </row>
     <row r="10" spans="2:65" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B10" s="69"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="73"/>
-      <c r="E10" s="74"/>
-      <c r="F10" s="74"/>
-      <c r="G10" s="74"/>
-      <c r="H10" s="75"/>
-      <c r="I10" s="73"/>
-      <c r="J10" s="74"/>
-      <c r="K10" s="74"/>
-      <c r="L10" s="74"/>
-      <c r="M10" s="74"/>
-      <c r="N10" s="74"/>
-      <c r="O10" s="74"/>
-      <c r="P10" s="74"/>
-      <c r="Q10" s="74"/>
-      <c r="R10" s="74"/>
-      <c r="S10" s="74"/>
-      <c r="T10" s="74"/>
-      <c r="U10" s="75"/>
-      <c r="V10" s="54"/>
-      <c r="W10" s="54"/>
-      <c r="X10" s="54"/>
-      <c r="Y10" s="54"/>
-      <c r="Z10" s="54"/>
-      <c r="AA10" s="54"/>
-      <c r="AB10" s="54"/>
-      <c r="AC10" s="54"/>
-      <c r="AD10" s="54"/>
-      <c r="AE10" s="54"/>
-      <c r="AF10" s="54"/>
-      <c r="AG10" s="54"/>
-      <c r="AH10" s="54"/>
-      <c r="AI10" s="54"/>
-      <c r="AJ10" s="54"/>
-      <c r="AK10" s="54"/>
-      <c r="AL10" s="54"/>
-      <c r="AM10" s="54"/>
-      <c r="AN10" s="54"/>
-      <c r="AO10" s="54"/>
-      <c r="AP10" s="54"/>
-      <c r="AQ10" s="54"/>
-      <c r="AR10" s="54"/>
-      <c r="AS10" s="54"/>
-      <c r="AT10" s="54"/>
-      <c r="AU10" s="54"/>
-      <c r="AV10" s="54"/>
-      <c r="AW10" s="54"/>
-      <c r="AX10" s="54"/>
-      <c r="AY10" s="54"/>
-      <c r="AZ10" s="54"/>
-      <c r="BA10" s="54"/>
-      <c r="BB10" s="54"/>
-      <c r="BC10" s="57"/>
-      <c r="BD10" s="57"/>
-      <c r="BE10" s="57"/>
-      <c r="BF10" s="57"/>
-      <c r="BG10" s="57"/>
-      <c r="BH10" s="57"/>
-      <c r="BI10" s="57"/>
-      <c r="BJ10" s="57"/>
-      <c r="BK10" s="57"/>
-      <c r="BL10" s="57"/>
-      <c r="BM10" s="58"/>
+      <c r="B10" s="89"/>
+      <c r="C10" s="81"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="94"/>
+      <c r="F10" s="94"/>
+      <c r="G10" s="94"/>
+      <c r="H10" s="95"/>
+      <c r="I10" s="93"/>
+      <c r="J10" s="94"/>
+      <c r="K10" s="94"/>
+      <c r="L10" s="94"/>
+      <c r="M10" s="94"/>
+      <c r="N10" s="94"/>
+      <c r="O10" s="94"/>
+      <c r="P10" s="94"/>
+      <c r="Q10" s="94"/>
+      <c r="R10" s="94"/>
+      <c r="S10" s="94"/>
+      <c r="T10" s="94"/>
+      <c r="U10" s="95"/>
+      <c r="V10" s="78"/>
+      <c r="W10" s="78"/>
+      <c r="X10" s="78"/>
+      <c r="Y10" s="78"/>
+      <c r="Z10" s="78"/>
+      <c r="AA10" s="78"/>
+      <c r="AB10" s="78"/>
+      <c r="AC10" s="78"/>
+      <c r="AD10" s="78"/>
+      <c r="AE10" s="78"/>
+      <c r="AF10" s="78"/>
+      <c r="AG10" s="78"/>
+      <c r="AH10" s="78"/>
+      <c r="AI10" s="78"/>
+      <c r="AJ10" s="78"/>
+      <c r="AK10" s="78"/>
+      <c r="AL10" s="78"/>
+      <c r="AM10" s="78"/>
+      <c r="AN10" s="78"/>
+      <c r="AO10" s="78"/>
+      <c r="AP10" s="78"/>
+      <c r="AQ10" s="78"/>
+      <c r="AR10" s="78"/>
+      <c r="AS10" s="78"/>
+      <c r="AT10" s="78"/>
+      <c r="AU10" s="78"/>
+      <c r="AV10" s="78"/>
+      <c r="AW10" s="78"/>
+      <c r="AX10" s="78"/>
+      <c r="AY10" s="78"/>
+      <c r="AZ10" s="78"/>
+      <c r="BA10" s="78"/>
+      <c r="BB10" s="78"/>
+      <c r="BC10" s="81"/>
+      <c r="BD10" s="81"/>
+      <c r="BE10" s="81"/>
+      <c r="BF10" s="81"/>
+      <c r="BG10" s="81"/>
+      <c r="BH10" s="81"/>
+      <c r="BI10" s="81"/>
+      <c r="BJ10" s="81"/>
+      <c r="BK10" s="81"/>
+      <c r="BL10" s="81"/>
+      <c r="BM10" s="82"/>
     </row>
     <row r="11" spans="2:65" ht="30" customHeight="1" thickTop="1">
-      <c r="B11" s="59">
+      <c r="B11" s="83">
         <v>1</v>
       </c>
-      <c r="C11" s="60"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="62"/>
-      <c r="F11" s="62"/>
-      <c r="G11" s="62"/>
-      <c r="H11" s="63"/>
-      <c r="I11" s="64"/>
-      <c r="J11" s="65"/>
-      <c r="K11" s="65"/>
-      <c r="L11" s="65"/>
-      <c r="M11" s="65"/>
-      <c r="N11" s="65"/>
-      <c r="O11" s="65"/>
-      <c r="P11" s="65"/>
-      <c r="Q11" s="65"/>
-      <c r="R11" s="65"/>
-      <c r="S11" s="65"/>
-      <c r="T11" s="65"/>
-      <c r="U11" s="66"/>
-      <c r="V11" s="64"/>
-      <c r="W11" s="65"/>
-      <c r="X11" s="65"/>
-      <c r="Y11" s="65"/>
-      <c r="Z11" s="65"/>
-      <c r="AA11" s="65"/>
-      <c r="AB11" s="65"/>
-      <c r="AC11" s="65"/>
-      <c r="AD11" s="65"/>
-      <c r="AE11" s="65"/>
-      <c r="AF11" s="65"/>
-      <c r="AG11" s="66"/>
-      <c r="AH11" s="64"/>
-      <c r="AI11" s="65"/>
-      <c r="AJ11" s="66"/>
-      <c r="AK11" s="64"/>
-      <c r="AL11" s="65"/>
-      <c r="AM11" s="66"/>
-      <c r="AN11" s="67"/>
-      <c r="AO11" s="67"/>
-      <c r="AP11" s="67"/>
-      <c r="AQ11" s="67"/>
-      <c r="AR11" s="67"/>
-      <c r="AS11" s="67"/>
-      <c r="AT11" s="67"/>
-      <c r="AU11" s="67"/>
-      <c r="AV11" s="67"/>
-      <c r="AW11" s="67"/>
-      <c r="AX11" s="67"/>
-      <c r="AY11" s="67"/>
-      <c r="AZ11" s="67"/>
-      <c r="BA11" s="67"/>
-      <c r="BB11" s="67"/>
-      <c r="BC11" s="67"/>
-      <c r="BD11" s="67"/>
-      <c r="BE11" s="67"/>
-      <c r="BF11" s="67"/>
-      <c r="BG11" s="67"/>
-      <c r="BH11" s="67"/>
-      <c r="BI11" s="67"/>
-      <c r="BJ11" s="67"/>
-      <c r="BK11" s="67"/>
-      <c r="BL11" s="67"/>
-      <c r="BM11" s="76"/>
+      <c r="C11" s="84"/>
+      <c r="D11" s="85"/>
+      <c r="E11" s="86"/>
+      <c r="F11" s="86"/>
+      <c r="G11" s="86"/>
+      <c r="H11" s="87"/>
+      <c r="I11" s="69"/>
+      <c r="J11" s="70"/>
+      <c r="K11" s="70"/>
+      <c r="L11" s="70"/>
+      <c r="M11" s="70"/>
+      <c r="N11" s="70"/>
+      <c r="O11" s="70"/>
+      <c r="P11" s="70"/>
+      <c r="Q11" s="70"/>
+      <c r="R11" s="70"/>
+      <c r="S11" s="70"/>
+      <c r="T11" s="70"/>
+      <c r="U11" s="71"/>
+      <c r="V11" s="69"/>
+      <c r="W11" s="70"/>
+      <c r="X11" s="70"/>
+      <c r="Y11" s="70"/>
+      <c r="Z11" s="70"/>
+      <c r="AA11" s="70"/>
+      <c r="AB11" s="70"/>
+      <c r="AC11" s="70"/>
+      <c r="AD11" s="70"/>
+      <c r="AE11" s="70"/>
+      <c r="AF11" s="70"/>
+      <c r="AG11" s="71"/>
+      <c r="AH11" s="69"/>
+      <c r="AI11" s="70"/>
+      <c r="AJ11" s="71"/>
+      <c r="AK11" s="69"/>
+      <c r="AL11" s="70"/>
+      <c r="AM11" s="71"/>
+      <c r="AN11" s="75"/>
+      <c r="AO11" s="75"/>
+      <c r="AP11" s="75"/>
+      <c r="AQ11" s="75"/>
+      <c r="AR11" s="75"/>
+      <c r="AS11" s="75"/>
+      <c r="AT11" s="75"/>
+      <c r="AU11" s="75"/>
+      <c r="AV11" s="75"/>
+      <c r="AW11" s="75"/>
+      <c r="AX11" s="75"/>
+      <c r="AY11" s="75"/>
+      <c r="AZ11" s="75"/>
+      <c r="BA11" s="75"/>
+      <c r="BB11" s="75"/>
+      <c r="BC11" s="75"/>
+      <c r="BD11" s="75"/>
+      <c r="BE11" s="75"/>
+      <c r="BF11" s="75"/>
+      <c r="BG11" s="75"/>
+      <c r="BH11" s="75"/>
+      <c r="BI11" s="75"/>
+      <c r="BJ11" s="75"/>
+      <c r="BK11" s="75"/>
+      <c r="BL11" s="75"/>
+      <c r="BM11" s="96"/>
     </row>
     <row r="12" spans="2:65" ht="30" customHeight="1">
-      <c r="B12" s="77">
+      <c r="B12" s="56">
         <f t="shared" ref="B12:B18" si="0">B11+1</f>
         <v>2</v>
       </c>
-      <c r="C12" s="78"/>
-      <c r="D12" s="79"/>
-      <c r="E12" s="80"/>
-      <c r="F12" s="80"/>
-      <c r="G12" s="80"/>
-      <c r="H12" s="81"/>
-      <c r="I12" s="64"/>
-      <c r="J12" s="65"/>
-      <c r="K12" s="65"/>
-      <c r="L12" s="65"/>
-      <c r="M12" s="65"/>
-      <c r="N12" s="65"/>
-      <c r="O12" s="65"/>
-      <c r="P12" s="65"/>
-      <c r="Q12" s="65"/>
-      <c r="R12" s="65"/>
-      <c r="S12" s="65"/>
-      <c r="T12" s="65"/>
-      <c r="U12" s="66"/>
-      <c r="V12" s="64"/>
-      <c r="W12" s="65"/>
-      <c r="X12" s="65"/>
-      <c r="Y12" s="65"/>
-      <c r="Z12" s="65"/>
-      <c r="AA12" s="65"/>
-      <c r="AB12" s="65"/>
-      <c r="AC12" s="65"/>
-      <c r="AD12" s="65"/>
-      <c r="AE12" s="65"/>
-      <c r="AF12" s="65"/>
-      <c r="AG12" s="66"/>
-      <c r="AH12" s="64"/>
-      <c r="AI12" s="65"/>
-      <c r="AJ12" s="66"/>
-      <c r="AK12" s="64"/>
-      <c r="AL12" s="65"/>
-      <c r="AM12" s="66"/>
-      <c r="AN12" s="64"/>
-      <c r="AO12" s="65"/>
-      <c r="AP12" s="65"/>
-      <c r="AQ12" s="65"/>
-      <c r="AR12" s="65"/>
-      <c r="AS12" s="65"/>
-      <c r="AT12" s="66"/>
-      <c r="AU12" s="64"/>
-      <c r="AV12" s="65"/>
-      <c r="AW12" s="65"/>
-      <c r="AX12" s="65"/>
-      <c r="AY12" s="65"/>
-      <c r="AZ12" s="65"/>
-      <c r="BA12" s="65"/>
-      <c r="BB12" s="66"/>
-      <c r="BC12" s="64"/>
-      <c r="BD12" s="65"/>
-      <c r="BE12" s="65"/>
-      <c r="BF12" s="65"/>
-      <c r="BG12" s="65"/>
-      <c r="BH12" s="65"/>
-      <c r="BI12" s="65"/>
-      <c r="BJ12" s="65"/>
-      <c r="BK12" s="65"/>
-      <c r="BL12" s="65"/>
-      <c r="BM12" s="82"/>
+      <c r="C12" s="57"/>
+      <c r="D12" s="66"/>
+      <c r="E12" s="67"/>
+      <c r="F12" s="67"/>
+      <c r="G12" s="67"/>
+      <c r="H12" s="68"/>
+      <c r="I12" s="69"/>
+      <c r="J12" s="70"/>
+      <c r="K12" s="70"/>
+      <c r="L12" s="70"/>
+      <c r="M12" s="70"/>
+      <c r="N12" s="70"/>
+      <c r="O12" s="70"/>
+      <c r="P12" s="70"/>
+      <c r="Q12" s="70"/>
+      <c r="R12" s="70"/>
+      <c r="S12" s="70"/>
+      <c r="T12" s="70"/>
+      <c r="U12" s="71"/>
+      <c r="V12" s="69"/>
+      <c r="W12" s="70"/>
+      <c r="X12" s="70"/>
+      <c r="Y12" s="70"/>
+      <c r="Z12" s="70"/>
+      <c r="AA12" s="70"/>
+      <c r="AB12" s="70"/>
+      <c r="AC12" s="70"/>
+      <c r="AD12" s="70"/>
+      <c r="AE12" s="70"/>
+      <c r="AF12" s="70"/>
+      <c r="AG12" s="71"/>
+      <c r="AH12" s="69"/>
+      <c r="AI12" s="70"/>
+      <c r="AJ12" s="71"/>
+      <c r="AK12" s="69"/>
+      <c r="AL12" s="70"/>
+      <c r="AM12" s="71"/>
+      <c r="AN12" s="69"/>
+      <c r="AO12" s="70"/>
+      <c r="AP12" s="70"/>
+      <c r="AQ12" s="70"/>
+      <c r="AR12" s="70"/>
+      <c r="AS12" s="70"/>
+      <c r="AT12" s="71"/>
+      <c r="AU12" s="69"/>
+      <c r="AV12" s="70"/>
+      <c r="AW12" s="70"/>
+      <c r="AX12" s="70"/>
+      <c r="AY12" s="70"/>
+      <c r="AZ12" s="70"/>
+      <c r="BA12" s="70"/>
+      <c r="BB12" s="71"/>
+      <c r="BC12" s="69"/>
+      <c r="BD12" s="70"/>
+      <c r="BE12" s="70"/>
+      <c r="BF12" s="70"/>
+      <c r="BG12" s="70"/>
+      <c r="BH12" s="70"/>
+      <c r="BI12" s="70"/>
+      <c r="BJ12" s="70"/>
+      <c r="BK12" s="70"/>
+      <c r="BL12" s="70"/>
+      <c r="BM12" s="76"/>
     </row>
     <row r="13" spans="2:65" ht="30" customHeight="1">
-      <c r="B13" s="77">
+      <c r="B13" s="56">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C13" s="78"/>
-      <c r="D13" s="79"/>
-      <c r="E13" s="80"/>
-      <c r="F13" s="80"/>
-      <c r="G13" s="80"/>
-      <c r="H13" s="81"/>
-      <c r="I13" s="64"/>
-      <c r="J13" s="65"/>
-      <c r="K13" s="65"/>
-      <c r="L13" s="65"/>
-      <c r="M13" s="65"/>
-      <c r="N13" s="65"/>
-      <c r="O13" s="65"/>
-      <c r="P13" s="65"/>
-      <c r="Q13" s="65"/>
-      <c r="R13" s="65"/>
-      <c r="S13" s="65"/>
-      <c r="T13" s="65"/>
-      <c r="U13" s="66"/>
-      <c r="V13" s="64"/>
-      <c r="W13" s="65"/>
-      <c r="X13" s="65"/>
-      <c r="Y13" s="65"/>
-      <c r="Z13" s="65"/>
-      <c r="AA13" s="65"/>
-      <c r="AB13" s="65"/>
-      <c r="AC13" s="65"/>
-      <c r="AD13" s="65"/>
-      <c r="AE13" s="65"/>
-      <c r="AF13" s="65"/>
-      <c r="AG13" s="66"/>
-      <c r="AH13" s="64"/>
-      <c r="AI13" s="65"/>
-      <c r="AJ13" s="66"/>
-      <c r="AK13" s="64"/>
-      <c r="AL13" s="65"/>
-      <c r="AM13" s="66"/>
-      <c r="AN13" s="64"/>
-      <c r="AO13" s="65"/>
-      <c r="AP13" s="65"/>
-      <c r="AQ13" s="65"/>
-      <c r="AR13" s="65"/>
-      <c r="AS13" s="65"/>
-      <c r="AT13" s="66"/>
-      <c r="AU13" s="64"/>
-      <c r="AV13" s="65"/>
-      <c r="AW13" s="65"/>
-      <c r="AX13" s="65"/>
-      <c r="AY13" s="65"/>
-      <c r="AZ13" s="65"/>
-      <c r="BA13" s="65"/>
-      <c r="BB13" s="66"/>
-      <c r="BC13" s="64"/>
-      <c r="BD13" s="65"/>
-      <c r="BE13" s="65"/>
-      <c r="BF13" s="65"/>
-      <c r="BG13" s="65"/>
-      <c r="BH13" s="65"/>
-      <c r="BI13" s="65"/>
-      <c r="BJ13" s="65"/>
-      <c r="BK13" s="65"/>
-      <c r="BL13" s="65"/>
-      <c r="BM13" s="82"/>
+      <c r="C13" s="57"/>
+      <c r="D13" s="66"/>
+      <c r="E13" s="67"/>
+      <c r="F13" s="67"/>
+      <c r="G13" s="67"/>
+      <c r="H13" s="68"/>
+      <c r="I13" s="69"/>
+      <c r="J13" s="70"/>
+      <c r="K13" s="70"/>
+      <c r="L13" s="70"/>
+      <c r="M13" s="70"/>
+      <c r="N13" s="70"/>
+      <c r="O13" s="70"/>
+      <c r="P13" s="70"/>
+      <c r="Q13" s="70"/>
+      <c r="R13" s="70"/>
+      <c r="S13" s="70"/>
+      <c r="T13" s="70"/>
+      <c r="U13" s="71"/>
+      <c r="V13" s="69"/>
+      <c r="W13" s="70"/>
+      <c r="X13" s="70"/>
+      <c r="Y13" s="70"/>
+      <c r="Z13" s="70"/>
+      <c r="AA13" s="70"/>
+      <c r="AB13" s="70"/>
+      <c r="AC13" s="70"/>
+      <c r="AD13" s="70"/>
+      <c r="AE13" s="70"/>
+      <c r="AF13" s="70"/>
+      <c r="AG13" s="71"/>
+      <c r="AH13" s="69"/>
+      <c r="AI13" s="70"/>
+      <c r="AJ13" s="71"/>
+      <c r="AK13" s="69"/>
+      <c r="AL13" s="70"/>
+      <c r="AM13" s="71"/>
+      <c r="AN13" s="69"/>
+      <c r="AO13" s="70"/>
+      <c r="AP13" s="70"/>
+      <c r="AQ13" s="70"/>
+      <c r="AR13" s="70"/>
+      <c r="AS13" s="70"/>
+      <c r="AT13" s="71"/>
+      <c r="AU13" s="69"/>
+      <c r="AV13" s="70"/>
+      <c r="AW13" s="70"/>
+      <c r="AX13" s="70"/>
+      <c r="AY13" s="70"/>
+      <c r="AZ13" s="70"/>
+      <c r="BA13" s="70"/>
+      <c r="BB13" s="71"/>
+      <c r="BC13" s="69"/>
+      <c r="BD13" s="70"/>
+      <c r="BE13" s="70"/>
+      <c r="BF13" s="70"/>
+      <c r="BG13" s="70"/>
+      <c r="BH13" s="70"/>
+      <c r="BI13" s="70"/>
+      <c r="BJ13" s="70"/>
+      <c r="BK13" s="70"/>
+      <c r="BL13" s="70"/>
+      <c r="BM13" s="76"/>
     </row>
     <row r="14" spans="2:65" ht="30" customHeight="1">
-      <c r="B14" s="77">
+      <c r="B14" s="56">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C14" s="78"/>
-      <c r="D14" s="79"/>
-      <c r="E14" s="80"/>
-      <c r="F14" s="80"/>
-      <c r="G14" s="80"/>
-      <c r="H14" s="81"/>
-      <c r="I14" s="64"/>
-      <c r="J14" s="65"/>
-      <c r="K14" s="65"/>
-      <c r="L14" s="65"/>
-      <c r="M14" s="65"/>
-      <c r="N14" s="65"/>
-      <c r="O14" s="65"/>
-      <c r="P14" s="65"/>
-      <c r="Q14" s="65"/>
-      <c r="R14" s="65"/>
-      <c r="S14" s="65"/>
-      <c r="T14" s="65"/>
-      <c r="U14" s="66"/>
-      <c r="V14" s="64"/>
-      <c r="W14" s="65"/>
-      <c r="X14" s="65"/>
-      <c r="Y14" s="65"/>
-      <c r="Z14" s="65"/>
-      <c r="AA14" s="65"/>
-      <c r="AB14" s="65"/>
-      <c r="AC14" s="65"/>
-      <c r="AD14" s="65"/>
-      <c r="AE14" s="65"/>
-      <c r="AF14" s="65"/>
-      <c r="AG14" s="66"/>
-      <c r="AH14" s="64"/>
-      <c r="AI14" s="65"/>
-      <c r="AJ14" s="66"/>
-      <c r="AK14" s="64"/>
-      <c r="AL14" s="65"/>
-      <c r="AM14" s="66"/>
-      <c r="AN14" s="64"/>
-      <c r="AO14" s="65"/>
-      <c r="AP14" s="65"/>
-      <c r="AQ14" s="65"/>
-      <c r="AR14" s="65"/>
-      <c r="AS14" s="65"/>
-      <c r="AT14" s="66"/>
-      <c r="AU14" s="64"/>
-      <c r="AV14" s="65"/>
-      <c r="AW14" s="65"/>
-      <c r="AX14" s="65"/>
-      <c r="AY14" s="65"/>
-      <c r="AZ14" s="65"/>
-      <c r="BA14" s="65"/>
-      <c r="BB14" s="66"/>
-      <c r="BC14" s="64"/>
-      <c r="BD14" s="65"/>
-      <c r="BE14" s="65"/>
-      <c r="BF14" s="65"/>
-      <c r="BG14" s="65"/>
-      <c r="BH14" s="65"/>
-      <c r="BI14" s="65"/>
-      <c r="BJ14" s="65"/>
-      <c r="BK14" s="65"/>
-      <c r="BL14" s="65"/>
-      <c r="BM14" s="82"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="66"/>
+      <c r="E14" s="67"/>
+      <c r="F14" s="67"/>
+      <c r="G14" s="67"/>
+      <c r="H14" s="68"/>
+      <c r="I14" s="69"/>
+      <c r="J14" s="70"/>
+      <c r="K14" s="70"/>
+      <c r="L14" s="70"/>
+      <c r="M14" s="70"/>
+      <c r="N14" s="70"/>
+      <c r="O14" s="70"/>
+      <c r="P14" s="70"/>
+      <c r="Q14" s="70"/>
+      <c r="R14" s="70"/>
+      <c r="S14" s="70"/>
+      <c r="T14" s="70"/>
+      <c r="U14" s="71"/>
+      <c r="V14" s="69"/>
+      <c r="W14" s="70"/>
+      <c r="X14" s="70"/>
+      <c r="Y14" s="70"/>
+      <c r="Z14" s="70"/>
+      <c r="AA14" s="70"/>
+      <c r="AB14" s="70"/>
+      <c r="AC14" s="70"/>
+      <c r="AD14" s="70"/>
+      <c r="AE14" s="70"/>
+      <c r="AF14" s="70"/>
+      <c r="AG14" s="71"/>
+      <c r="AH14" s="69"/>
+      <c r="AI14" s="70"/>
+      <c r="AJ14" s="71"/>
+      <c r="AK14" s="69"/>
+      <c r="AL14" s="70"/>
+      <c r="AM14" s="71"/>
+      <c r="AN14" s="69"/>
+      <c r="AO14" s="70"/>
+      <c r="AP14" s="70"/>
+      <c r="AQ14" s="70"/>
+      <c r="AR14" s="70"/>
+      <c r="AS14" s="70"/>
+      <c r="AT14" s="71"/>
+      <c r="AU14" s="69"/>
+      <c r="AV14" s="70"/>
+      <c r="AW14" s="70"/>
+      <c r="AX14" s="70"/>
+      <c r="AY14" s="70"/>
+      <c r="AZ14" s="70"/>
+      <c r="BA14" s="70"/>
+      <c r="BB14" s="71"/>
+      <c r="BC14" s="69"/>
+      <c r="BD14" s="70"/>
+      <c r="BE14" s="70"/>
+      <c r="BF14" s="70"/>
+      <c r="BG14" s="70"/>
+      <c r="BH14" s="70"/>
+      <c r="BI14" s="70"/>
+      <c r="BJ14" s="70"/>
+      <c r="BK14" s="70"/>
+      <c r="BL14" s="70"/>
+      <c r="BM14" s="76"/>
     </row>
     <row r="15" spans="2:65" ht="30" customHeight="1">
-      <c r="B15" s="77">
+      <c r="B15" s="56">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C15" s="78"/>
-      <c r="D15" s="79"/>
-      <c r="E15" s="80"/>
-      <c r="F15" s="80"/>
-      <c r="G15" s="80"/>
-      <c r="H15" s="81"/>
-      <c r="I15" s="64"/>
-      <c r="J15" s="65"/>
-      <c r="K15" s="65"/>
-      <c r="L15" s="65"/>
-      <c r="M15" s="65"/>
-      <c r="N15" s="65"/>
-      <c r="O15" s="65"/>
-      <c r="P15" s="65"/>
-      <c r="Q15" s="65"/>
-      <c r="R15" s="65"/>
-      <c r="S15" s="65"/>
-      <c r="T15" s="65"/>
-      <c r="U15" s="66"/>
-      <c r="V15" s="64"/>
-      <c r="W15" s="65"/>
-      <c r="X15" s="65"/>
-      <c r="Y15" s="65"/>
-      <c r="Z15" s="65"/>
-      <c r="AA15" s="65"/>
-      <c r="AB15" s="65"/>
-      <c r="AC15" s="65"/>
-      <c r="AD15" s="65"/>
-      <c r="AE15" s="65"/>
-      <c r="AF15" s="65"/>
-      <c r="AG15" s="66"/>
-      <c r="AH15" s="64"/>
-      <c r="AI15" s="65"/>
-      <c r="AJ15" s="66"/>
-      <c r="AK15" s="64"/>
-      <c r="AL15" s="65"/>
-      <c r="AM15" s="66"/>
-      <c r="AN15" s="64"/>
-      <c r="AO15" s="65"/>
-      <c r="AP15" s="65"/>
-      <c r="AQ15" s="65"/>
-      <c r="AR15" s="65"/>
-      <c r="AS15" s="65"/>
-      <c r="AT15" s="66"/>
-      <c r="AU15" s="64"/>
-      <c r="AV15" s="65"/>
-      <c r="AW15" s="65"/>
-      <c r="AX15" s="65"/>
-      <c r="AY15" s="65"/>
-      <c r="AZ15" s="65"/>
-      <c r="BA15" s="65"/>
-      <c r="BB15" s="66"/>
-      <c r="BC15" s="64"/>
-      <c r="BD15" s="65"/>
-      <c r="BE15" s="65"/>
-      <c r="BF15" s="65"/>
-      <c r="BG15" s="65"/>
-      <c r="BH15" s="65"/>
-      <c r="BI15" s="65"/>
-      <c r="BJ15" s="65"/>
-      <c r="BK15" s="65"/>
-      <c r="BL15" s="65"/>
-      <c r="BM15" s="82"/>
+      <c r="C15" s="57"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="67"/>
+      <c r="F15" s="67"/>
+      <c r="G15" s="67"/>
+      <c r="H15" s="68"/>
+      <c r="I15" s="69"/>
+      <c r="J15" s="70"/>
+      <c r="K15" s="70"/>
+      <c r="L15" s="70"/>
+      <c r="M15" s="70"/>
+      <c r="N15" s="70"/>
+      <c r="O15" s="70"/>
+      <c r="P15" s="70"/>
+      <c r="Q15" s="70"/>
+      <c r="R15" s="70"/>
+      <c r="S15" s="70"/>
+      <c r="T15" s="70"/>
+      <c r="U15" s="71"/>
+      <c r="V15" s="69"/>
+      <c r="W15" s="70"/>
+      <c r="X15" s="70"/>
+      <c r="Y15" s="70"/>
+      <c r="Z15" s="70"/>
+      <c r="AA15" s="70"/>
+      <c r="AB15" s="70"/>
+      <c r="AC15" s="70"/>
+      <c r="AD15" s="70"/>
+      <c r="AE15" s="70"/>
+      <c r="AF15" s="70"/>
+      <c r="AG15" s="71"/>
+      <c r="AH15" s="69"/>
+      <c r="AI15" s="70"/>
+      <c r="AJ15" s="71"/>
+      <c r="AK15" s="69"/>
+      <c r="AL15" s="70"/>
+      <c r="AM15" s="71"/>
+      <c r="AN15" s="69"/>
+      <c r="AO15" s="70"/>
+      <c r="AP15" s="70"/>
+      <c r="AQ15" s="70"/>
+      <c r="AR15" s="70"/>
+      <c r="AS15" s="70"/>
+      <c r="AT15" s="71"/>
+      <c r="AU15" s="69"/>
+      <c r="AV15" s="70"/>
+      <c r="AW15" s="70"/>
+      <c r="AX15" s="70"/>
+      <c r="AY15" s="70"/>
+      <c r="AZ15" s="70"/>
+      <c r="BA15" s="70"/>
+      <c r="BB15" s="71"/>
+      <c r="BC15" s="69"/>
+      <c r="BD15" s="70"/>
+      <c r="BE15" s="70"/>
+      <c r="BF15" s="70"/>
+      <c r="BG15" s="70"/>
+      <c r="BH15" s="70"/>
+      <c r="BI15" s="70"/>
+      <c r="BJ15" s="70"/>
+      <c r="BK15" s="70"/>
+      <c r="BL15" s="70"/>
+      <c r="BM15" s="76"/>
     </row>
     <row r="16" spans="2:65" ht="30" customHeight="1">
-      <c r="B16" s="77">
+      <c r="B16" s="56">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C16" s="78"/>
-      <c r="D16" s="79"/>
-      <c r="E16" s="80"/>
-      <c r="F16" s="80"/>
-      <c r="G16" s="80"/>
-      <c r="H16" s="81"/>
-      <c r="I16" s="64"/>
-      <c r="J16" s="65"/>
-      <c r="K16" s="65"/>
-      <c r="L16" s="65"/>
-      <c r="M16" s="65"/>
-      <c r="N16" s="65"/>
-      <c r="O16" s="65"/>
-      <c r="P16" s="65"/>
-      <c r="Q16" s="65"/>
-      <c r="R16" s="65"/>
-      <c r="S16" s="65"/>
-      <c r="T16" s="65"/>
-      <c r="U16" s="66"/>
-      <c r="V16" s="64"/>
-      <c r="W16" s="65"/>
-      <c r="X16" s="65"/>
-      <c r="Y16" s="65"/>
-      <c r="Z16" s="65"/>
-      <c r="AA16" s="65"/>
-      <c r="AB16" s="65"/>
-      <c r="AC16" s="65"/>
-      <c r="AD16" s="65"/>
-      <c r="AE16" s="65"/>
-      <c r="AF16" s="65"/>
-      <c r="AG16" s="66"/>
-      <c r="AH16" s="64"/>
-      <c r="AI16" s="65"/>
-      <c r="AJ16" s="66"/>
-      <c r="AK16" s="64"/>
-      <c r="AL16" s="65"/>
-      <c r="AM16" s="66"/>
-      <c r="AN16" s="83"/>
-      <c r="AO16" s="84"/>
-      <c r="AP16" s="84"/>
-      <c r="AQ16" s="84"/>
-      <c r="AR16" s="84"/>
-      <c r="AS16" s="84"/>
-      <c r="AT16" s="85"/>
-      <c r="AU16" s="67"/>
-      <c r="AV16" s="67"/>
-      <c r="AW16" s="67"/>
-      <c r="AX16" s="67"/>
-      <c r="AY16" s="67"/>
-      <c r="AZ16" s="67"/>
-      <c r="BA16" s="67"/>
-      <c r="BB16" s="67"/>
-      <c r="BC16" s="64"/>
-      <c r="BD16" s="65"/>
-      <c r="BE16" s="65"/>
-      <c r="BF16" s="65"/>
-      <c r="BG16" s="65"/>
-      <c r="BH16" s="65"/>
-      <c r="BI16" s="65"/>
-      <c r="BJ16" s="65"/>
-      <c r="BK16" s="65"/>
-      <c r="BL16" s="65"/>
-      <c r="BM16" s="82"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="67"/>
+      <c r="F16" s="67"/>
+      <c r="G16" s="67"/>
+      <c r="H16" s="68"/>
+      <c r="I16" s="69"/>
+      <c r="J16" s="70"/>
+      <c r="K16" s="70"/>
+      <c r="L16" s="70"/>
+      <c r="M16" s="70"/>
+      <c r="N16" s="70"/>
+      <c r="O16" s="70"/>
+      <c r="P16" s="70"/>
+      <c r="Q16" s="70"/>
+      <c r="R16" s="70"/>
+      <c r="S16" s="70"/>
+      <c r="T16" s="70"/>
+      <c r="U16" s="71"/>
+      <c r="V16" s="69"/>
+      <c r="W16" s="70"/>
+      <c r="X16" s="70"/>
+      <c r="Y16" s="70"/>
+      <c r="Z16" s="70"/>
+      <c r="AA16" s="70"/>
+      <c r="AB16" s="70"/>
+      <c r="AC16" s="70"/>
+      <c r="AD16" s="70"/>
+      <c r="AE16" s="70"/>
+      <c r="AF16" s="70"/>
+      <c r="AG16" s="71"/>
+      <c r="AH16" s="69"/>
+      <c r="AI16" s="70"/>
+      <c r="AJ16" s="71"/>
+      <c r="AK16" s="69"/>
+      <c r="AL16" s="70"/>
+      <c r="AM16" s="71"/>
+      <c r="AN16" s="72"/>
+      <c r="AO16" s="73"/>
+      <c r="AP16" s="73"/>
+      <c r="AQ16" s="73"/>
+      <c r="AR16" s="73"/>
+      <c r="AS16" s="73"/>
+      <c r="AT16" s="74"/>
+      <c r="AU16" s="75"/>
+      <c r="AV16" s="75"/>
+      <c r="AW16" s="75"/>
+      <c r="AX16" s="75"/>
+      <c r="AY16" s="75"/>
+      <c r="AZ16" s="75"/>
+      <c r="BA16" s="75"/>
+      <c r="BB16" s="75"/>
+      <c r="BC16" s="69"/>
+      <c r="BD16" s="70"/>
+      <c r="BE16" s="70"/>
+      <c r="BF16" s="70"/>
+      <c r="BG16" s="70"/>
+      <c r="BH16" s="70"/>
+      <c r="BI16" s="70"/>
+      <c r="BJ16" s="70"/>
+      <c r="BK16" s="70"/>
+      <c r="BL16" s="70"/>
+      <c r="BM16" s="76"/>
     </row>
     <row r="17" spans="2:65" ht="30" customHeight="1">
-      <c r="B17" s="77">
+      <c r="B17" s="56">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C17" s="78"/>
-      <c r="D17" s="79"/>
-      <c r="E17" s="80"/>
-      <c r="F17" s="80"/>
-      <c r="G17" s="80"/>
-      <c r="H17" s="81"/>
-      <c r="I17" s="64"/>
-      <c r="J17" s="65"/>
-      <c r="K17" s="65"/>
-      <c r="L17" s="65"/>
-      <c r="M17" s="65"/>
-      <c r="N17" s="65"/>
-      <c r="O17" s="65"/>
-      <c r="P17" s="65"/>
-      <c r="Q17" s="65"/>
-      <c r="R17" s="65"/>
-      <c r="S17" s="65"/>
-      <c r="T17" s="65"/>
-      <c r="U17" s="66"/>
-      <c r="V17" s="64"/>
-      <c r="W17" s="65"/>
-      <c r="X17" s="65"/>
-      <c r="Y17" s="65"/>
-      <c r="Z17" s="65"/>
-      <c r="AA17" s="65"/>
-      <c r="AB17" s="65"/>
-      <c r="AC17" s="65"/>
-      <c r="AD17" s="65"/>
-      <c r="AE17" s="65"/>
-      <c r="AF17" s="65"/>
-      <c r="AG17" s="66"/>
-      <c r="AH17" s="64"/>
-      <c r="AI17" s="65"/>
-      <c r="AJ17" s="66"/>
-      <c r="AK17" s="64"/>
-      <c r="AL17" s="65"/>
-      <c r="AM17" s="66"/>
-      <c r="AN17" s="83"/>
-      <c r="AO17" s="84"/>
-      <c r="AP17" s="84"/>
-      <c r="AQ17" s="84"/>
-      <c r="AR17" s="84"/>
-      <c r="AS17" s="84"/>
-      <c r="AT17" s="85"/>
-      <c r="AU17" s="67"/>
-      <c r="AV17" s="67"/>
-      <c r="AW17" s="67"/>
-      <c r="AX17" s="67"/>
-      <c r="AY17" s="67"/>
-      <c r="AZ17" s="67"/>
-      <c r="BA17" s="67"/>
-      <c r="BB17" s="67"/>
-      <c r="BC17" s="64"/>
-      <c r="BD17" s="65"/>
-      <c r="BE17" s="65"/>
-      <c r="BF17" s="65"/>
-      <c r="BG17" s="65"/>
-      <c r="BH17" s="65"/>
-      <c r="BI17" s="65"/>
-      <c r="BJ17" s="65"/>
-      <c r="BK17" s="65"/>
-      <c r="BL17" s="65"/>
-      <c r="BM17" s="82"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="67"/>
+      <c r="F17" s="67"/>
+      <c r="G17" s="67"/>
+      <c r="H17" s="68"/>
+      <c r="I17" s="69"/>
+      <c r="J17" s="70"/>
+      <c r="K17" s="70"/>
+      <c r="L17" s="70"/>
+      <c r="M17" s="70"/>
+      <c r="N17" s="70"/>
+      <c r="O17" s="70"/>
+      <c r="P17" s="70"/>
+      <c r="Q17" s="70"/>
+      <c r="R17" s="70"/>
+      <c r="S17" s="70"/>
+      <c r="T17" s="70"/>
+      <c r="U17" s="71"/>
+      <c r="V17" s="69"/>
+      <c r="W17" s="70"/>
+      <c r="X17" s="70"/>
+      <c r="Y17" s="70"/>
+      <c r="Z17" s="70"/>
+      <c r="AA17" s="70"/>
+      <c r="AB17" s="70"/>
+      <c r="AC17" s="70"/>
+      <c r="AD17" s="70"/>
+      <c r="AE17" s="70"/>
+      <c r="AF17" s="70"/>
+      <c r="AG17" s="71"/>
+      <c r="AH17" s="69"/>
+      <c r="AI17" s="70"/>
+      <c r="AJ17" s="71"/>
+      <c r="AK17" s="69"/>
+      <c r="AL17" s="70"/>
+      <c r="AM17" s="71"/>
+      <c r="AN17" s="72"/>
+      <c r="AO17" s="73"/>
+      <c r="AP17" s="73"/>
+      <c r="AQ17" s="73"/>
+      <c r="AR17" s="73"/>
+      <c r="AS17" s="73"/>
+      <c r="AT17" s="74"/>
+      <c r="AU17" s="75"/>
+      <c r="AV17" s="75"/>
+      <c r="AW17" s="75"/>
+      <c r="AX17" s="75"/>
+      <c r="AY17" s="75"/>
+      <c r="AZ17" s="75"/>
+      <c r="BA17" s="75"/>
+      <c r="BB17" s="75"/>
+      <c r="BC17" s="69"/>
+      <c r="BD17" s="70"/>
+      <c r="BE17" s="70"/>
+      <c r="BF17" s="70"/>
+      <c r="BG17" s="70"/>
+      <c r="BH17" s="70"/>
+      <c r="BI17" s="70"/>
+      <c r="BJ17" s="70"/>
+      <c r="BK17" s="70"/>
+      <c r="BL17" s="70"/>
+      <c r="BM17" s="76"/>
     </row>
     <row r="18" spans="2:65" ht="30" customHeight="1" thickBot="1">
-      <c r="B18" s="77">
+      <c r="B18" s="56">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C18" s="78"/>
-      <c r="D18" s="106"/>
-      <c r="E18" s="107"/>
-      <c r="F18" s="107"/>
-      <c r="G18" s="107"/>
-      <c r="H18" s="108"/>
-      <c r="I18" s="109"/>
-      <c r="J18" s="110"/>
-      <c r="K18" s="110"/>
-      <c r="L18" s="110"/>
-      <c r="M18" s="110"/>
-      <c r="N18" s="110"/>
-      <c r="O18" s="110"/>
-      <c r="P18" s="110"/>
-      <c r="Q18" s="110"/>
-      <c r="R18" s="110"/>
-      <c r="S18" s="110"/>
-      <c r="T18" s="110"/>
-      <c r="U18" s="111"/>
-      <c r="V18" s="112"/>
-      <c r="W18" s="112"/>
-      <c r="X18" s="112"/>
-      <c r="Y18" s="112"/>
-      <c r="Z18" s="112"/>
-      <c r="AA18" s="112"/>
-      <c r="AB18" s="112"/>
-      <c r="AC18" s="112"/>
-      <c r="AD18" s="112"/>
-      <c r="AE18" s="112"/>
-      <c r="AF18" s="112"/>
-      <c r="AG18" s="112"/>
-      <c r="AH18" s="112"/>
-      <c r="AI18" s="112"/>
-      <c r="AJ18" s="112"/>
-      <c r="AK18" s="112"/>
-      <c r="AL18" s="112"/>
-      <c r="AM18" s="112"/>
-      <c r="AN18" s="95"/>
-      <c r="AO18" s="95"/>
-      <c r="AP18" s="95"/>
-      <c r="AQ18" s="95"/>
-      <c r="AR18" s="95"/>
-      <c r="AS18" s="95"/>
-      <c r="AT18" s="95"/>
-      <c r="AU18" s="95"/>
-      <c r="AV18" s="95"/>
-      <c r="AW18" s="95"/>
-      <c r="AX18" s="95"/>
-      <c r="AY18" s="95"/>
-      <c r="AZ18" s="95"/>
-      <c r="BA18" s="95"/>
-      <c r="BB18" s="95"/>
-      <c r="BC18" s="95"/>
-      <c r="BD18" s="95"/>
-      <c r="BE18" s="95"/>
-      <c r="BF18" s="95"/>
-      <c r="BG18" s="95"/>
-      <c r="BH18" s="95"/>
-      <c r="BI18" s="95"/>
-      <c r="BJ18" s="95"/>
-      <c r="BK18" s="95"/>
-      <c r="BL18" s="95"/>
-      <c r="BM18" s="96"/>
+      <c r="C18" s="57"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="59"/>
+      <c r="F18" s="59"/>
+      <c r="G18" s="59"/>
+      <c r="H18" s="60"/>
+      <c r="I18" s="61"/>
+      <c r="J18" s="62"/>
+      <c r="K18" s="62"/>
+      <c r="L18" s="62"/>
+      <c r="M18" s="62"/>
+      <c r="N18" s="62"/>
+      <c r="O18" s="62"/>
+      <c r="P18" s="62"/>
+      <c r="Q18" s="62"/>
+      <c r="R18" s="62"/>
+      <c r="S18" s="62"/>
+      <c r="T18" s="62"/>
+      <c r="U18" s="63"/>
+      <c r="V18" s="64"/>
+      <c r="W18" s="64"/>
+      <c r="X18" s="64"/>
+      <c r="Y18" s="64"/>
+      <c r="Z18" s="64"/>
+      <c r="AA18" s="64"/>
+      <c r="AB18" s="64"/>
+      <c r="AC18" s="64"/>
+      <c r="AD18" s="64"/>
+      <c r="AE18" s="64"/>
+      <c r="AF18" s="64"/>
+      <c r="AG18" s="64"/>
+      <c r="AH18" s="64"/>
+      <c r="AI18" s="64"/>
+      <c r="AJ18" s="64"/>
+      <c r="AK18" s="64"/>
+      <c r="AL18" s="64"/>
+      <c r="AM18" s="64"/>
+      <c r="AN18" s="45"/>
+      <c r="AO18" s="45"/>
+      <c r="AP18" s="45"/>
+      <c r="AQ18" s="45"/>
+      <c r="AR18" s="45"/>
+      <c r="AS18" s="45"/>
+      <c r="AT18" s="45"/>
+      <c r="AU18" s="45"/>
+      <c r="AV18" s="45"/>
+      <c r="AW18" s="45"/>
+      <c r="AX18" s="45"/>
+      <c r="AY18" s="45"/>
+      <c r="AZ18" s="45"/>
+      <c r="BA18" s="45"/>
+      <c r="BB18" s="45"/>
+      <c r="BC18" s="45"/>
+      <c r="BD18" s="45"/>
+      <c r="BE18" s="45"/>
+      <c r="BF18" s="45"/>
+      <c r="BG18" s="45"/>
+      <c r="BH18" s="45"/>
+      <c r="BI18" s="45"/>
+      <c r="BJ18" s="45"/>
+      <c r="BK18" s="45"/>
+      <c r="BL18" s="45"/>
+      <c r="BM18" s="46"/>
     </row>
     <row r="19" spans="2:65" ht="15.75" thickTop="1" thickBot="1">
       <c r="B19" s="12"/>
@@ -2852,206 +2864,206 @@
       <c r="BM19" s="16"/>
     </row>
     <row r="20" spans="2:65" ht="15.75" customHeight="1" thickTop="1">
-      <c r="B20" s="97" t="s">
+      <c r="B20" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="98"/>
-      <c r="D20" s="98"/>
-      <c r="E20" s="98"/>
-      <c r="F20" s="98"/>
-      <c r="G20" s="98"/>
-      <c r="H20" s="98"/>
-      <c r="I20" s="98"/>
-      <c r="J20" s="98"/>
-      <c r="K20" s="98"/>
-      <c r="L20" s="98"/>
-      <c r="M20" s="98"/>
-      <c r="N20" s="98"/>
-      <c r="O20" s="98"/>
-      <c r="P20" s="98"/>
-      <c r="Q20" s="98"/>
-      <c r="R20" s="98"/>
-      <c r="S20" s="98"/>
-      <c r="T20" s="98"/>
-      <c r="U20" s="98"/>
-      <c r="V20" s="98"/>
-      <c r="W20" s="98"/>
-      <c r="X20" s="98"/>
-      <c r="Y20" s="98"/>
-      <c r="Z20" s="98"/>
-      <c r="AA20" s="98"/>
-      <c r="AB20" s="98"/>
-      <c r="AC20" s="98"/>
-      <c r="AD20" s="98"/>
-      <c r="AE20" s="98"/>
-      <c r="AF20" s="98"/>
-      <c r="AG20" s="98"/>
-      <c r="AH20" s="98"/>
-      <c r="AI20" s="98"/>
-      <c r="AJ20" s="98"/>
-      <c r="AK20" s="98"/>
-      <c r="AL20" s="98"/>
-      <c r="AM20" s="98"/>
-      <c r="AN20" s="98"/>
-      <c r="AO20" s="99"/>
-      <c r="AP20" s="100" t="s">
+      <c r="C20" s="48"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="48"/>
+      <c r="F20" s="48"/>
+      <c r="G20" s="48"/>
+      <c r="H20" s="48"/>
+      <c r="I20" s="48"/>
+      <c r="J20" s="48"/>
+      <c r="K20" s="48"/>
+      <c r="L20" s="48"/>
+      <c r="M20" s="48"/>
+      <c r="N20" s="48"/>
+      <c r="O20" s="48"/>
+      <c r="P20" s="48"/>
+      <c r="Q20" s="48"/>
+      <c r="R20" s="48"/>
+      <c r="S20" s="48"/>
+      <c r="T20" s="48"/>
+      <c r="U20" s="48"/>
+      <c r="V20" s="48"/>
+      <c r="W20" s="48"/>
+      <c r="X20" s="48"/>
+      <c r="Y20" s="48"/>
+      <c r="Z20" s="48"/>
+      <c r="AA20" s="48"/>
+      <c r="AB20" s="48"/>
+      <c r="AC20" s="48"/>
+      <c r="AD20" s="48"/>
+      <c r="AE20" s="48"/>
+      <c r="AF20" s="48"/>
+      <c r="AG20" s="48"/>
+      <c r="AH20" s="48"/>
+      <c r="AI20" s="48"/>
+      <c r="AJ20" s="48"/>
+      <c r="AK20" s="48"/>
+      <c r="AL20" s="48"/>
+      <c r="AM20" s="48"/>
+      <c r="AN20" s="48"/>
+      <c r="AO20" s="49"/>
+      <c r="AP20" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="AQ20" s="101"/>
-      <c r="AR20" s="101"/>
-      <c r="AS20" s="101"/>
-      <c r="AT20" s="101"/>
-      <c r="AU20" s="101"/>
-      <c r="AV20" s="101"/>
-      <c r="AW20" s="101"/>
-      <c r="AX20" s="101"/>
-      <c r="AY20" s="101"/>
-      <c r="AZ20" s="101"/>
-      <c r="BA20" s="101"/>
-      <c r="BB20" s="101"/>
-      <c r="BC20" s="101"/>
-      <c r="BD20" s="101"/>
-      <c r="BE20" s="101"/>
-      <c r="BF20" s="101"/>
-      <c r="BG20" s="101"/>
-      <c r="BH20" s="101"/>
-      <c r="BI20" s="101"/>
-      <c r="BJ20" s="101"/>
-      <c r="BK20" s="101"/>
-      <c r="BL20" s="101"/>
-      <c r="BM20" s="102"/>
+      <c r="AQ20" s="51"/>
+      <c r="AR20" s="51"/>
+      <c r="AS20" s="51"/>
+      <c r="AT20" s="51"/>
+      <c r="AU20" s="51"/>
+      <c r="AV20" s="51"/>
+      <c r="AW20" s="51"/>
+      <c r="AX20" s="51"/>
+      <c r="AY20" s="51"/>
+      <c r="AZ20" s="51"/>
+      <c r="BA20" s="51"/>
+      <c r="BB20" s="51"/>
+      <c r="BC20" s="51"/>
+      <c r="BD20" s="51"/>
+      <c r="BE20" s="51"/>
+      <c r="BF20" s="51"/>
+      <c r="BG20" s="51"/>
+      <c r="BH20" s="51"/>
+      <c r="BI20" s="51"/>
+      <c r="BJ20" s="51"/>
+      <c r="BK20" s="51"/>
+      <c r="BL20" s="51"/>
+      <c r="BM20" s="52"/>
     </row>
     <row r="21" spans="2:65" ht="15" customHeight="1">
       <c r="B21" s="22"/>
-      <c r="C21" s="121"/>
-      <c r="D21" s="121"/>
-      <c r="E21" s="121"/>
-      <c r="F21" s="121"/>
-      <c r="G21" s="121"/>
-      <c r="H21" s="121"/>
-      <c r="I21" s="121"/>
-      <c r="J21" s="121"/>
-      <c r="K21" s="121"/>
-      <c r="L21" s="121"/>
-      <c r="M21" s="121"/>
-      <c r="N21" s="121"/>
-      <c r="O21" s="121"/>
-      <c r="P21" s="121"/>
-      <c r="Q21" s="121"/>
-      <c r="R21" s="121"/>
-      <c r="S21" s="121"/>
-      <c r="T21" s="121"/>
-      <c r="U21" s="121"/>
-      <c r="V21" s="121"/>
-      <c r="W21" s="121"/>
-      <c r="X21" s="121"/>
-      <c r="Y21" s="121"/>
-      <c r="Z21" s="121"/>
-      <c r="AA21" s="121"/>
-      <c r="AB21" s="121"/>
-      <c r="AC21" s="121"/>
-      <c r="AD21" s="121"/>
-      <c r="AE21" s="121"/>
-      <c r="AF21" s="121"/>
-      <c r="AG21" s="121"/>
-      <c r="AH21" s="121"/>
-      <c r="AI21" s="121"/>
-      <c r="AJ21" s="121"/>
-      <c r="AK21" s="121"/>
-      <c r="AL21" s="121"/>
-      <c r="AM21" s="121"/>
-      <c r="AN21" s="121"/>
+      <c r="C21" s="65"/>
+      <c r="D21" s="65"/>
+      <c r="E21" s="65"/>
+      <c r="F21" s="65"/>
+      <c r="G21" s="65"/>
+      <c r="H21" s="65"/>
+      <c r="I21" s="65"/>
+      <c r="J21" s="65"/>
+      <c r="K21" s="65"/>
+      <c r="L21" s="65"/>
+      <c r="M21" s="65"/>
+      <c r="N21" s="65"/>
+      <c r="O21" s="65"/>
+      <c r="P21" s="65"/>
+      <c r="Q21" s="65"/>
+      <c r="R21" s="65"/>
+      <c r="S21" s="65"/>
+      <c r="T21" s="65"/>
+      <c r="U21" s="65"/>
+      <c r="V21" s="65"/>
+      <c r="W21" s="65"/>
+      <c r="X21" s="65"/>
+      <c r="Y21" s="65"/>
+      <c r="Z21" s="65"/>
+      <c r="AA21" s="65"/>
+      <c r="AB21" s="65"/>
+      <c r="AC21" s="65"/>
+      <c r="AD21" s="65"/>
+      <c r="AE21" s="65"/>
+      <c r="AF21" s="65"/>
+      <c r="AG21" s="65"/>
+      <c r="AH21" s="65"/>
+      <c r="AI21" s="65"/>
+      <c r="AJ21" s="65"/>
+      <c r="AK21" s="65"/>
+      <c r="AL21" s="65"/>
+      <c r="AM21" s="65"/>
+      <c r="AN21" s="65"/>
       <c r="AO21" s="23"/>
-      <c r="AP21" s="103"/>
-      <c r="AQ21" s="104"/>
-      <c r="AR21" s="104"/>
-      <c r="AS21" s="104"/>
-      <c r="AT21" s="104"/>
-      <c r="AU21" s="104"/>
-      <c r="AV21" s="104"/>
-      <c r="AW21" s="104"/>
-      <c r="AX21" s="104"/>
-      <c r="AY21" s="104"/>
-      <c r="AZ21" s="104"/>
-      <c r="BA21" s="104"/>
-      <c r="BB21" s="104"/>
-      <c r="BC21" s="104"/>
-      <c r="BD21" s="104"/>
-      <c r="BE21" s="104"/>
-      <c r="BF21" s="104"/>
-      <c r="BG21" s="104"/>
-      <c r="BH21" s="104"/>
-      <c r="BI21" s="104"/>
-      <c r="BJ21" s="104"/>
-      <c r="BK21" s="104"/>
-      <c r="BL21" s="104"/>
-      <c r="BM21" s="105"/>
+      <c r="AP21" s="53"/>
+      <c r="AQ21" s="54"/>
+      <c r="AR21" s="54"/>
+      <c r="AS21" s="54"/>
+      <c r="AT21" s="54"/>
+      <c r="AU21" s="54"/>
+      <c r="AV21" s="54"/>
+      <c r="AW21" s="54"/>
+      <c r="AX21" s="54"/>
+      <c r="AY21" s="54"/>
+      <c r="AZ21" s="54"/>
+      <c r="BA21" s="54"/>
+      <c r="BB21" s="54"/>
+      <c r="BC21" s="54"/>
+      <c r="BD21" s="54"/>
+      <c r="BE21" s="54"/>
+      <c r="BF21" s="54"/>
+      <c r="BG21" s="54"/>
+      <c r="BH21" s="54"/>
+      <c r="BI21" s="54"/>
+      <c r="BJ21" s="54"/>
+      <c r="BK21" s="54"/>
+      <c r="BL21" s="54"/>
+      <c r="BM21" s="55"/>
     </row>
     <row r="22" spans="2:65" ht="15" customHeight="1">
       <c r="B22" s="22"/>
-      <c r="C22" s="121"/>
-      <c r="D22" s="121"/>
-      <c r="E22" s="121"/>
-      <c r="F22" s="121"/>
-      <c r="G22" s="121"/>
-      <c r="H22" s="121"/>
-      <c r="I22" s="121"/>
-      <c r="J22" s="121"/>
-      <c r="K22" s="121"/>
-      <c r="L22" s="121"/>
-      <c r="M22" s="121"/>
-      <c r="N22" s="121"/>
-      <c r="O22" s="121"/>
-      <c r="P22" s="121"/>
-      <c r="Q22" s="121"/>
-      <c r="R22" s="121"/>
-      <c r="S22" s="121"/>
-      <c r="T22" s="121"/>
-      <c r="U22" s="121"/>
-      <c r="V22" s="121"/>
-      <c r="W22" s="121"/>
-      <c r="X22" s="121"/>
-      <c r="Y22" s="121"/>
-      <c r="Z22" s="121"/>
-      <c r="AA22" s="121"/>
-      <c r="AB22" s="121"/>
-      <c r="AC22" s="121"/>
-      <c r="AD22" s="121"/>
-      <c r="AE22" s="121"/>
-      <c r="AF22" s="121"/>
-      <c r="AG22" s="121"/>
-      <c r="AH22" s="121"/>
-      <c r="AI22" s="121"/>
-      <c r="AJ22" s="121"/>
-      <c r="AK22" s="121"/>
-      <c r="AL22" s="121"/>
-      <c r="AM22" s="121"/>
-      <c r="AN22" s="121"/>
+      <c r="C22" s="65"/>
+      <c r="D22" s="65"/>
+      <c r="E22" s="65"/>
+      <c r="F22" s="65"/>
+      <c r="G22" s="65"/>
+      <c r="H22" s="65"/>
+      <c r="I22" s="65"/>
+      <c r="J22" s="65"/>
+      <c r="K22" s="65"/>
+      <c r="L22" s="65"/>
+      <c r="M22" s="65"/>
+      <c r="N22" s="65"/>
+      <c r="O22" s="65"/>
+      <c r="P22" s="65"/>
+      <c r="Q22" s="65"/>
+      <c r="R22" s="65"/>
+      <c r="S22" s="65"/>
+      <c r="T22" s="65"/>
+      <c r="U22" s="65"/>
+      <c r="V22" s="65"/>
+      <c r="W22" s="65"/>
+      <c r="X22" s="65"/>
+      <c r="Y22" s="65"/>
+      <c r="Z22" s="65"/>
+      <c r="AA22" s="65"/>
+      <c r="AB22" s="65"/>
+      <c r="AC22" s="65"/>
+      <c r="AD22" s="65"/>
+      <c r="AE22" s="65"/>
+      <c r="AF22" s="65"/>
+      <c r="AG22" s="65"/>
+      <c r="AH22" s="65"/>
+      <c r="AI22" s="65"/>
+      <c r="AJ22" s="65"/>
+      <c r="AK22" s="65"/>
+      <c r="AL22" s="65"/>
+      <c r="AM22" s="65"/>
+      <c r="AN22" s="65"/>
       <c r="AO22" s="23"/>
-      <c r="AP22" s="86"/>
-      <c r="AQ22" s="87"/>
-      <c r="AR22" s="87"/>
-      <c r="AS22" s="87"/>
-      <c r="AT22" s="87"/>
-      <c r="AU22" s="87"/>
-      <c r="AV22" s="87"/>
-      <c r="AW22" s="87"/>
-      <c r="AX22" s="87"/>
-      <c r="AY22" s="87"/>
-      <c r="AZ22" s="87"/>
-      <c r="BA22" s="87"/>
-      <c r="BB22" s="87"/>
-      <c r="BC22" s="87"/>
-      <c r="BD22" s="87"/>
-      <c r="BE22" s="87"/>
-      <c r="BF22" s="87"/>
-      <c r="BG22" s="87"/>
-      <c r="BH22" s="87"/>
-      <c r="BI22" s="87"/>
-      <c r="BJ22" s="87"/>
-      <c r="BK22" s="87"/>
-      <c r="BL22" s="87"/>
-      <c r="BM22" s="88"/>
+      <c r="AP22" s="36"/>
+      <c r="AQ22" s="37"/>
+      <c r="AR22" s="37"/>
+      <c r="AS22" s="37"/>
+      <c r="AT22" s="37"/>
+      <c r="AU22" s="37"/>
+      <c r="AV22" s="37"/>
+      <c r="AW22" s="37"/>
+      <c r="AX22" s="37"/>
+      <c r="AY22" s="37"/>
+      <c r="AZ22" s="37"/>
+      <c r="BA22" s="37"/>
+      <c r="BB22" s="37"/>
+      <c r="BC22" s="37"/>
+      <c r="BD22" s="37"/>
+      <c r="BE22" s="37"/>
+      <c r="BF22" s="37"/>
+      <c r="BG22" s="37"/>
+      <c r="BH22" s="37"/>
+      <c r="BI22" s="37"/>
+      <c r="BJ22" s="37"/>
+      <c r="BK22" s="37"/>
+      <c r="BL22" s="37"/>
+      <c r="BM22" s="38"/>
     </row>
     <row r="23" spans="2:65" ht="15" customHeight="1" thickBot="1">
       <c r="B23" s="24"/>
@@ -3094,30 +3106,30 @@
       <c r="AM23" s="25"/>
       <c r="AN23" s="25"/>
       <c r="AO23" s="26"/>
-      <c r="AP23" s="89"/>
-      <c r="AQ23" s="90"/>
-      <c r="AR23" s="90"/>
-      <c r="AS23" s="90"/>
-      <c r="AT23" s="90"/>
-      <c r="AU23" s="90"/>
-      <c r="AV23" s="90"/>
-      <c r="AW23" s="90"/>
-      <c r="AX23" s="90"/>
-      <c r="AY23" s="90"/>
-      <c r="AZ23" s="90"/>
-      <c r="BA23" s="90"/>
-      <c r="BB23" s="90"/>
-      <c r="BC23" s="90"/>
-      <c r="BD23" s="90"/>
-      <c r="BE23" s="90"/>
-      <c r="BF23" s="90"/>
-      <c r="BG23" s="90"/>
-      <c r="BH23" s="90"/>
-      <c r="BI23" s="90"/>
-      <c r="BJ23" s="90"/>
-      <c r="BK23" s="90"/>
-      <c r="BL23" s="90"/>
-      <c r="BM23" s="91"/>
+      <c r="AP23" s="39"/>
+      <c r="AQ23" s="40"/>
+      <c r="AR23" s="40"/>
+      <c r="AS23" s="40"/>
+      <c r="AT23" s="40"/>
+      <c r="AU23" s="40"/>
+      <c r="AV23" s="40"/>
+      <c r="AW23" s="40"/>
+      <c r="AX23" s="40"/>
+      <c r="AY23" s="40"/>
+      <c r="AZ23" s="40"/>
+      <c r="BA23" s="40"/>
+      <c r="BB23" s="40"/>
+      <c r="BC23" s="40"/>
+      <c r="BD23" s="40"/>
+      <c r="BE23" s="40"/>
+      <c r="BF23" s="40"/>
+      <c r="BG23" s="40"/>
+      <c r="BH23" s="40"/>
+      <c r="BI23" s="40"/>
+      <c r="BJ23" s="40"/>
+      <c r="BK23" s="40"/>
+      <c r="BL23" s="40"/>
+      <c r="BM23" s="41"/>
     </row>
     <row r="24" spans="2:65" ht="15.75" thickTop="1" thickBot="1">
       <c r="B24" s="12"/>
@@ -3186,106 +3198,90 @@
       <c r="BM24" s="16"/>
     </row>
     <row r="25" spans="2:65" ht="16.5" thickTop="1" thickBot="1">
-      <c r="B25" s="92" t="s">
+      <c r="B25" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="93"/>
-      <c r="D25" s="93"/>
-      <c r="E25" s="93"/>
-      <c r="F25" s="93"/>
-      <c r="G25" s="93"/>
-      <c r="H25" s="93"/>
-      <c r="I25" s="93"/>
-      <c r="J25" s="93"/>
-      <c r="K25" s="93"/>
-      <c r="L25" s="93"/>
-      <c r="M25" s="94"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="43"/>
+      <c r="F25" s="43"/>
+      <c r="G25" s="43"/>
+      <c r="H25" s="43"/>
+      <c r="I25" s="43"/>
+      <c r="J25" s="43"/>
+      <c r="K25" s="43"/>
+      <c r="L25" s="43"/>
+      <c r="M25" s="44"/>
       <c r="N25" s="12"/>
-      <c r="O25" s="12"/>
-      <c r="P25" s="12"/>
-      <c r="Q25" s="12"/>
-      <c r="R25" s="12"/>
-      <c r="S25" s="12"/>
-      <c r="T25" s="12"/>
-      <c r="U25" s="12"/>
-      <c r="V25" s="12"/>
-      <c r="W25" s="12"/>
-      <c r="X25" s="12"/>
-      <c r="Y25" s="12"/>
-      <c r="Z25" s="12"/>
+      <c r="O25" s="42" t="s">
+        <v>30</v>
+      </c>
+      <c r="P25" s="43"/>
+      <c r="Q25" s="43"/>
+      <c r="R25" s="43"/>
+      <c r="S25" s="43"/>
+      <c r="T25" s="43"/>
+      <c r="U25" s="43"/>
+      <c r="V25" s="43"/>
+      <c r="W25" s="43"/>
+      <c r="X25" s="43"/>
+      <c r="Y25" s="43"/>
+      <c r="Z25" s="44"/>
       <c r="AA25" s="12"/>
-      <c r="AB25" s="92" t="s">
-        <v>29</v>
+      <c r="AB25" s="42" t="s">
+        <v>31</v>
       </c>
-      <c r="AC25" s="93"/>
-      <c r="AD25" s="93"/>
-      <c r="AE25" s="93"/>
-      <c r="AF25" s="93"/>
-      <c r="AG25" s="93"/>
-      <c r="AH25" s="93"/>
-      <c r="AI25" s="93"/>
-      <c r="AJ25" s="93"/>
-      <c r="AK25" s="93"/>
-      <c r="AL25" s="93"/>
-      <c r="AM25" s="94"/>
+      <c r="AC25" s="43"/>
+      <c r="AD25" s="43"/>
+      <c r="AE25" s="43"/>
+      <c r="AF25" s="43"/>
+      <c r="AG25" s="43"/>
+      <c r="AH25" s="43"/>
+      <c r="AI25" s="43"/>
+      <c r="AJ25" s="43"/>
+      <c r="AK25" s="43"/>
+      <c r="AL25" s="43"/>
+      <c r="AM25" s="44"/>
       <c r="AN25" s="16"/>
-      <c r="AO25" s="16"/>
-      <c r="AP25" s="16"/>
-      <c r="AQ25" s="16"/>
-      <c r="AR25" s="16"/>
-      <c r="AS25" s="16"/>
-      <c r="AT25" s="16"/>
-      <c r="AU25" s="16"/>
-      <c r="AV25" s="16"/>
-      <c r="AW25" s="16"/>
-      <c r="AX25" s="16"/>
-      <c r="AY25" s="16"/>
-      <c r="AZ25" s="16"/>
+      <c r="AO25" s="42" t="s">
+        <v>32</v>
+      </c>
+      <c r="AP25" s="43"/>
+      <c r="AQ25" s="43"/>
+      <c r="AR25" s="43"/>
+      <c r="AS25" s="43"/>
+      <c r="AT25" s="43"/>
+      <c r="AU25" s="43"/>
+      <c r="AV25" s="43"/>
+      <c r="AW25" s="43"/>
+      <c r="AX25" s="43"/>
+      <c r="AY25" s="43"/>
+      <c r="AZ25" s="44"/>
       <c r="BA25" s="16"/>
-      <c r="BB25" s="92" t="s">
+      <c r="BB25" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="BC25" s="93"/>
-      <c r="BD25" s="93"/>
-      <c r="BE25" s="93"/>
-      <c r="BF25" s="93"/>
-      <c r="BG25" s="93"/>
-      <c r="BH25" s="93"/>
-      <c r="BI25" s="93"/>
-      <c r="BJ25" s="93"/>
-      <c r="BK25" s="93"/>
-      <c r="BL25" s="93"/>
-      <c r="BM25" s="94"/>
+      <c r="BC25" s="43"/>
+      <c r="BD25" s="43"/>
+      <c r="BE25" s="43"/>
+      <c r="BF25" s="43"/>
+      <c r="BG25" s="43"/>
+      <c r="BH25" s="43"/>
+      <c r="BI25" s="43"/>
+      <c r="BJ25" s="43"/>
+      <c r="BK25" s="43"/>
+      <c r="BL25" s="43"/>
+      <c r="BM25" s="44"/>
     </row>
     <row r="26" spans="2:65" ht="15" thickTop="1">
       <c r="B26" s="13"/>
       <c r="M26" s="17"/>
-      <c r="O26" s="12"/>
-      <c r="P26" s="12"/>
-      <c r="Q26" s="12"/>
-      <c r="R26" s="12"/>
-      <c r="S26" s="12"/>
-      <c r="T26" s="12"/>
-      <c r="U26" s="12"/>
-      <c r="V26" s="12"/>
-      <c r="W26" s="12"/>
-      <c r="X26" s="12"/>
-      <c r="Y26" s="12"/>
-      <c r="Z26" s="12"/>
+      <c r="O26" s="13"/>
+      <c r="Z26" s="17"/>
       <c r="AB26" s="13"/>
       <c r="AM26" s="17"/>
-      <c r="AO26" s="16"/>
-      <c r="AP26" s="16"/>
-      <c r="AQ26" s="16"/>
-      <c r="AR26" s="16"/>
-      <c r="AS26" s="16"/>
-      <c r="AT26" s="16"/>
-      <c r="AU26" s="16"/>
-      <c r="AV26" s="16"/>
-      <c r="AW26" s="16"/>
-      <c r="AX26" s="16"/>
-      <c r="AY26" s="16"/>
-      <c r="AZ26" s="16"/>
+      <c r="AO26" s="13"/>
+      <c r="AZ26" s="17"/>
       <c r="BA26" s="16"/>
       <c r="BB26" s="13"/>
       <c r="BM26" s="17"/>
@@ -3294,33 +3290,15 @@
       <c r="B27" s="13"/>
       <c r="E27" s="14"/>
       <c r="M27" s="17"/>
-      <c r="O27" s="12"/>
-      <c r="P27" s="12"/>
-      <c r="Q27" s="12"/>
-      <c r="R27" s="12"/>
-      <c r="S27" s="12"/>
-      <c r="T27" s="12"/>
-      <c r="U27" s="12"/>
-      <c r="V27" s="12"/>
-      <c r="W27" s="12"/>
-      <c r="X27" s="12"/>
-      <c r="Y27" s="12"/>
-      <c r="Z27" s="12"/>
+      <c r="O27" s="13"/>
+      <c r="R27" s="14"/>
+      <c r="Z27" s="17"/>
       <c r="AB27" s="13"/>
       <c r="AE27" s="14"/>
       <c r="AM27" s="17"/>
-      <c r="AO27" s="16"/>
-      <c r="AP27" s="16"/>
-      <c r="AQ27" s="16"/>
-      <c r="AR27" s="16"/>
-      <c r="AS27" s="16"/>
-      <c r="AT27" s="16"/>
-      <c r="AU27" s="16"/>
-      <c r="AV27" s="16"/>
-      <c r="AW27" s="16"/>
-      <c r="AX27" s="16"/>
-      <c r="AY27" s="16"/>
-      <c r="AZ27" s="16"/>
+      <c r="AO27" s="13"/>
+      <c r="AR27" s="14"/>
+      <c r="AZ27" s="17"/>
       <c r="BA27" s="16"/>
       <c r="BB27" s="13"/>
       <c r="BM27" s="17"/>
@@ -3331,336 +3309,270 @@
       <c r="E28" s="14"/>
       <c r="F28" s="14"/>
       <c r="M28" s="17"/>
-      <c r="O28" s="12"/>
-      <c r="P28" s="12"/>
-      <c r="Q28" s="12"/>
-      <c r="R28" s="12"/>
-      <c r="S28" s="12"/>
-      <c r="T28" s="12"/>
-      <c r="U28" s="12"/>
-      <c r="V28" s="12"/>
-      <c r="W28" s="12"/>
-      <c r="X28" s="12"/>
-      <c r="Y28" s="12"/>
-      <c r="Z28" s="12"/>
+      <c r="O28" s="15"/>
+      <c r="P28" s="14"/>
+      <c r="R28" s="14"/>
+      <c r="S28" s="14"/>
+      <c r="Z28" s="17"/>
       <c r="AB28" s="15"/>
       <c r="AC28" s="14"/>
       <c r="AE28" s="14"/>
       <c r="AF28" s="14"/>
       <c r="AM28" s="17"/>
-      <c r="AO28" s="16"/>
-      <c r="AP28" s="16"/>
-      <c r="AQ28" s="16"/>
-      <c r="AR28" s="16"/>
-      <c r="AS28" s="16"/>
-      <c r="AT28" s="16"/>
-      <c r="AU28" s="16"/>
-      <c r="AV28" s="16"/>
-      <c r="AW28" s="16"/>
-      <c r="AX28" s="16"/>
-      <c r="AY28" s="16"/>
-      <c r="AZ28" s="16"/>
+      <c r="AO28" s="15"/>
+      <c r="AP28" s="14"/>
+      <c r="AR28" s="14"/>
+      <c r="AS28" s="14"/>
+      <c r="AZ28" s="17"/>
       <c r="BA28" s="16"/>
       <c r="BB28" s="13"/>
       <c r="BM28" s="17"/>
     </row>
-    <row r="29" spans="2:65" ht="14.25" customHeight="1">
+    <row r="29" spans="2:65">
       <c r="B29" s="13"/>
       <c r="M29" s="17"/>
-      <c r="O29" s="12"/>
-      <c r="P29" s="12"/>
-      <c r="Q29" s="12"/>
-      <c r="R29" s="12"/>
-      <c r="S29" s="12"/>
-      <c r="T29" s="12"/>
-      <c r="U29" s="12"/>
-      <c r="V29" s="12"/>
-      <c r="W29" s="12"/>
-      <c r="X29" s="12"/>
-      <c r="Y29" s="12"/>
-      <c r="Z29" s="12"/>
+      <c r="O29" s="13"/>
+      <c r="Z29" s="17"/>
       <c r="AB29" s="13"/>
       <c r="AM29" s="17"/>
-      <c r="AO29" s="16"/>
-      <c r="AP29" s="16"/>
-      <c r="AQ29" s="16"/>
-      <c r="AR29" s="16"/>
-      <c r="AS29" s="16"/>
-      <c r="AT29" s="16"/>
-      <c r="AU29" s="16"/>
-      <c r="AV29" s="16"/>
-      <c r="AW29" s="16"/>
-      <c r="AX29" s="16"/>
-      <c r="AY29" s="16"/>
-      <c r="AZ29" s="16"/>
+      <c r="AO29" s="13"/>
+      <c r="AZ29" s="17"/>
       <c r="BA29" s="16"/>
       <c r="BB29" s="13"/>
       <c r="BM29" s="17"/>
     </row>
-    <row r="30" spans="2:65" ht="14.25" customHeight="1">
+    <row r="30" spans="2:65">
       <c r="B30" s="13"/>
       <c r="M30" s="17"/>
-      <c r="O30" s="12"/>
-      <c r="P30" s="12"/>
-      <c r="Q30" s="12"/>
-      <c r="R30" s="12"/>
-      <c r="S30" s="12"/>
-      <c r="T30" s="12"/>
-      <c r="U30" s="12"/>
-      <c r="V30" s="12"/>
-      <c r="W30" s="12"/>
-      <c r="X30" s="12"/>
-      <c r="Y30" s="12"/>
-      <c r="Z30" s="12"/>
+      <c r="O30" s="13"/>
+      <c r="Z30" s="17"/>
       <c r="AB30" s="13"/>
       <c r="AM30" s="17"/>
-      <c r="AO30" s="16"/>
-      <c r="AP30" s="16"/>
-      <c r="AQ30" s="16"/>
-      <c r="AR30" s="16"/>
-      <c r="AS30" s="16"/>
-      <c r="AT30" s="16"/>
-      <c r="AU30" s="16"/>
-      <c r="AV30" s="16"/>
-      <c r="AW30" s="16"/>
-      <c r="AX30" s="16"/>
-      <c r="AY30" s="16"/>
-      <c r="AZ30" s="16"/>
+      <c r="AO30" s="13"/>
+      <c r="AZ30" s="17"/>
       <c r="BA30" s="16"/>
       <c r="BB30" s="13"/>
       <c r="BM30" s="17"/>
     </row>
-    <row r="31" spans="2:65" ht="14.25" customHeight="1">
+    <row r="31" spans="2:65">
       <c r="B31" s="13"/>
       <c r="M31" s="17"/>
-      <c r="O31" s="12"/>
-      <c r="P31" s="12"/>
-      <c r="Q31" s="12"/>
-      <c r="R31" s="12"/>
-      <c r="S31" s="12"/>
-      <c r="T31" s="12"/>
-      <c r="U31" s="12"/>
-      <c r="V31" s="12"/>
-      <c r="W31" s="12"/>
-      <c r="X31" s="12"/>
-      <c r="Y31" s="12"/>
-      <c r="Z31" s="12"/>
+      <c r="O31" s="13"/>
+      <c r="Z31" s="17"/>
       <c r="AB31" s="13"/>
       <c r="AM31" s="17"/>
-      <c r="AO31" s="16"/>
-      <c r="AP31" s="16"/>
-      <c r="AQ31" s="16"/>
-      <c r="AR31" s="16"/>
-      <c r="AS31" s="16"/>
-      <c r="AT31" s="16"/>
-      <c r="AU31" s="16"/>
-      <c r="AV31" s="16"/>
-      <c r="AW31" s="16"/>
-      <c r="AX31" s="16"/>
-      <c r="AY31" s="16"/>
-      <c r="AZ31" s="16"/>
+      <c r="AO31" s="13"/>
+      <c r="AZ31" s="17"/>
       <c r="BA31" s="16"/>
       <c r="BB31" s="13"/>
       <c r="BM31" s="17"/>
     </row>
     <row r="32" spans="2:65" ht="14.25" customHeight="1">
-      <c r="B32" s="113"/>
-      <c r="C32" s="114"/>
-      <c r="D32" s="114"/>
-      <c r="E32" s="114"/>
-      <c r="F32" s="114"/>
-      <c r="G32" s="114"/>
-      <c r="H32" s="114"/>
-      <c r="I32" s="114"/>
-      <c r="J32" s="114"/>
-      <c r="K32" s="114"/>
-      <c r="L32" s="114"/>
-      <c r="M32" s="115"/>
-      <c r="O32" s="12"/>
-      <c r="P32" s="12"/>
-      <c r="Q32" s="12"/>
-      <c r="R32" s="12"/>
-      <c r="S32" s="12"/>
-      <c r="T32" s="12"/>
-      <c r="U32" s="12"/>
-      <c r="V32" s="12"/>
-      <c r="W32" s="12"/>
-      <c r="X32" s="12"/>
-      <c r="Y32" s="12"/>
-      <c r="Z32" s="12"/>
-      <c r="AB32" s="113"/>
-      <c r="AC32" s="114"/>
-      <c r="AD32" s="114"/>
-      <c r="AE32" s="114"/>
-      <c r="AF32" s="114"/>
-      <c r="AG32" s="114"/>
-      <c r="AH32" s="114"/>
-      <c r="AI32" s="114"/>
-      <c r="AJ32" s="114"/>
-      <c r="AK32" s="114"/>
-      <c r="AL32" s="114"/>
-      <c r="AM32" s="115"/>
-      <c r="AO32" s="16"/>
-      <c r="AP32" s="16"/>
-      <c r="AQ32" s="16"/>
-      <c r="AR32" s="16"/>
-      <c r="AS32" s="16"/>
-      <c r="AT32" s="16"/>
-      <c r="AU32" s="16"/>
-      <c r="AV32" s="16"/>
-      <c r="AW32" s="16"/>
-      <c r="AX32" s="16"/>
-      <c r="AY32" s="16"/>
-      <c r="AZ32" s="16"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="28"/>
+      <c r="K32" s="28"/>
+      <c r="L32" s="28"/>
+      <c r="M32" s="29"/>
+      <c r="O32" s="27"/>
+      <c r="P32" s="28"/>
+      <c r="Q32" s="28"/>
+      <c r="R32" s="28"/>
+      <c r="S32" s="28"/>
+      <c r="T32" s="28"/>
+      <c r="U32" s="28"/>
+      <c r="V32" s="28"/>
+      <c r="W32" s="28"/>
+      <c r="X32" s="28"/>
+      <c r="Y32" s="28"/>
+      <c r="Z32" s="29"/>
+      <c r="AB32" s="27"/>
+      <c r="AC32" s="28"/>
+      <c r="AD32" s="28"/>
+      <c r="AE32" s="28"/>
+      <c r="AF32" s="28"/>
+      <c r="AG32" s="28"/>
+      <c r="AH32" s="28"/>
+      <c r="AI32" s="28"/>
+      <c r="AJ32" s="28"/>
+      <c r="AK32" s="28"/>
+      <c r="AL32" s="28"/>
+      <c r="AM32" s="29"/>
+      <c r="AO32" s="27"/>
+      <c r="AP32" s="28"/>
+      <c r="AQ32" s="28"/>
+      <c r="AR32" s="28"/>
+      <c r="AS32" s="28"/>
+      <c r="AT32" s="28"/>
+      <c r="AU32" s="28"/>
+      <c r="AV32" s="28"/>
+      <c r="AW32" s="28"/>
+      <c r="AX32" s="28"/>
+      <c r="AY32" s="28"/>
+      <c r="AZ32" s="29"/>
       <c r="BA32" s="16"/>
-      <c r="BB32" s="113"/>
-      <c r="BC32" s="114"/>
-      <c r="BD32" s="114"/>
-      <c r="BE32" s="114"/>
-      <c r="BF32" s="114"/>
-      <c r="BG32" s="114"/>
-      <c r="BH32" s="114"/>
-      <c r="BI32" s="114"/>
-      <c r="BJ32" s="114"/>
-      <c r="BK32" s="114"/>
-      <c r="BL32" s="114"/>
-      <c r="BM32" s="115"/>
+      <c r="BB32" s="27"/>
+      <c r="BC32" s="28"/>
+      <c r="BD32" s="28"/>
+      <c r="BE32" s="28"/>
+      <c r="BF32" s="28"/>
+      <c r="BG32" s="28"/>
+      <c r="BH32" s="28"/>
+      <c r="BI32" s="28"/>
+      <c r="BJ32" s="28"/>
+      <c r="BK32" s="28"/>
+      <c r="BL32" s="28"/>
+      <c r="BM32" s="29"/>
     </row>
     <row r="33" spans="2:65" ht="14.25" customHeight="1">
-      <c r="B33" s="116"/>
-      <c r="C33" s="117"/>
-      <c r="D33" s="117"/>
-      <c r="E33" s="117"/>
-      <c r="F33" s="117"/>
-      <c r="G33" s="117"/>
-      <c r="H33" s="117"/>
-      <c r="I33" s="117"/>
-      <c r="J33" s="117"/>
-      <c r="K33" s="117"/>
-      <c r="L33" s="117"/>
-      <c r="M33" s="118"/>
-      <c r="O33" s="12"/>
-      <c r="P33" s="12"/>
-      <c r="Q33" s="12"/>
-      <c r="R33" s="12"/>
-      <c r="S33" s="12"/>
-      <c r="T33" s="12"/>
-      <c r="U33" s="12"/>
-      <c r="V33" s="12"/>
-      <c r="W33" s="12"/>
-      <c r="X33" s="12"/>
-      <c r="Y33" s="12"/>
-      <c r="Z33" s="12"/>
-      <c r="AB33" s="116" t="s">
+      <c r="B33" s="30"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="31"/>
+      <c r="F33" s="31"/>
+      <c r="G33" s="31"/>
+      <c r="H33" s="31"/>
+      <c r="I33" s="31"/>
+      <c r="J33" s="31"/>
+      <c r="K33" s="31"/>
+      <c r="L33" s="31"/>
+      <c r="M33" s="32"/>
+      <c r="O33" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="P33" s="31"/>
+      <c r="Q33" s="31"/>
+      <c r="R33" s="31"/>
+      <c r="S33" s="31"/>
+      <c r="T33" s="31"/>
+      <c r="U33" s="31"/>
+      <c r="V33" s="31"/>
+      <c r="W33" s="31"/>
+      <c r="X33" s="31"/>
+      <c r="Y33" s="31"/>
+      <c r="Z33" s="32"/>
+      <c r="AB33" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="AC33" s="117"/>
-      <c r="AD33" s="117"/>
-      <c r="AE33" s="117"/>
-      <c r="AF33" s="117"/>
-      <c r="AG33" s="117"/>
-      <c r="AH33" s="117"/>
-      <c r="AI33" s="117"/>
-      <c r="AJ33" s="117"/>
-      <c r="AK33" s="117"/>
-      <c r="AL33" s="117"/>
-      <c r="AM33" s="118"/>
-      <c r="AO33" s="16"/>
-      <c r="AP33" s="16"/>
-      <c r="AQ33" s="16"/>
-      <c r="AR33" s="16"/>
-      <c r="AS33" s="16"/>
-      <c r="AT33" s="16"/>
-      <c r="AU33" s="16"/>
-      <c r="AV33" s="16"/>
-      <c r="AW33" s="16"/>
-      <c r="AX33" s="16"/>
-      <c r="AY33" s="16"/>
-      <c r="AZ33" s="16"/>
+      <c r="AC33" s="31"/>
+      <c r="AD33" s="31"/>
+      <c r="AE33" s="31"/>
+      <c r="AF33" s="31"/>
+      <c r="AG33" s="31"/>
+      <c r="AH33" s="31"/>
+      <c r="AI33" s="31"/>
+      <c r="AJ33" s="31"/>
+      <c r="AK33" s="31"/>
+      <c r="AL33" s="31"/>
+      <c r="AM33" s="32"/>
+      <c r="AO33" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="AP33" s="31"/>
+      <c r="AQ33" s="31"/>
+      <c r="AR33" s="31"/>
+      <c r="AS33" s="31"/>
+      <c r="AT33" s="31"/>
+      <c r="AU33" s="31"/>
+      <c r="AV33" s="31"/>
+      <c r="AW33" s="31"/>
+      <c r="AX33" s="31"/>
+      <c r="AY33" s="31"/>
+      <c r="AZ33" s="32"/>
       <c r="BA33" s="16"/>
-      <c r="BB33" s="116" t="s">
+      <c r="BB33" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="BC33" s="117"/>
-      <c r="BD33" s="117"/>
-      <c r="BE33" s="117"/>
-      <c r="BF33" s="117"/>
-      <c r="BG33" s="117"/>
-      <c r="BH33" s="117"/>
-      <c r="BI33" s="117"/>
-      <c r="BJ33" s="117"/>
-      <c r="BK33" s="117"/>
-      <c r="BL33" s="117"/>
-      <c r="BM33" s="118"/>
+      <c r="BC33" s="31"/>
+      <c r="BD33" s="31"/>
+      <c r="BE33" s="31"/>
+      <c r="BF33" s="31"/>
+      <c r="BG33" s="31"/>
+      <c r="BH33" s="31"/>
+      <c r="BI33" s="31"/>
+      <c r="BJ33" s="31"/>
+      <c r="BK33" s="31"/>
+      <c r="BL33" s="31"/>
+      <c r="BM33" s="32"/>
     </row>
     <row r="34" spans="2:65" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B34" s="119" t="s">
+      <c r="B34" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="C34" s="120"/>
-      <c r="D34" s="120"/>
-      <c r="E34" s="120"/>
-      <c r="F34" s="120"/>
-      <c r="G34" s="120"/>
-      <c r="H34" s="120"/>
-      <c r="I34" s="120"/>
-      <c r="J34" s="120"/>
-      <c r="K34" s="120"/>
-      <c r="L34" s="120"/>
-      <c r="M34" s="122"/>
-      <c r="O34" s="12"/>
-      <c r="P34" s="12"/>
-      <c r="Q34" s="12"/>
-      <c r="R34" s="12"/>
-      <c r="S34" s="12"/>
-      <c r="T34" s="12"/>
-      <c r="U34" s="12"/>
-      <c r="V34" s="12"/>
-      <c r="W34" s="12"/>
-      <c r="X34" s="12"/>
-      <c r="Y34" s="12"/>
-      <c r="Z34" s="12"/>
-      <c r="AB34" s="119" t="s">
+      <c r="C34" s="34"/>
+      <c r="D34" s="34"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="34"/>
+      <c r="H34" s="34"/>
+      <c r="I34" s="34"/>
+      <c r="J34" s="34"/>
+      <c r="K34" s="34"/>
+      <c r="L34" s="34"/>
+      <c r="M34" s="35"/>
+      <c r="O34" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="AC34" s="120"/>
-      <c r="AD34" s="120"/>
-      <c r="AE34" s="120"/>
-      <c r="AF34" s="120"/>
-      <c r="AG34" s="120"/>
-      <c r="AH34" s="120"/>
-      <c r="AI34" s="120"/>
-      <c r="AJ34" s="120"/>
-      <c r="AK34" s="120"/>
-      <c r="AL34" s="120"/>
-      <c r="AM34" s="122"/>
-      <c r="AO34" s="16"/>
-      <c r="AP34" s="16"/>
-      <c r="AQ34" s="16"/>
-      <c r="AR34" s="16"/>
-      <c r="AS34" s="16"/>
-      <c r="AT34" s="16"/>
-      <c r="AU34" s="16"/>
-      <c r="AV34" s="16"/>
-      <c r="AW34" s="16"/>
-      <c r="AX34" s="16"/>
-      <c r="AY34" s="16"/>
-      <c r="AZ34" s="16"/>
-      <c r="BA34" s="16"/>
-      <c r="BB34" s="119" t="s">
+      <c r="P34" s="34"/>
+      <c r="Q34" s="34"/>
+      <c r="R34" s="34"/>
+      <c r="S34" s="34"/>
+      <c r="T34" s="34"/>
+      <c r="U34" s="34"/>
+      <c r="V34" s="34"/>
+      <c r="W34" s="34"/>
+      <c r="X34" s="34"/>
+      <c r="Y34" s="34"/>
+      <c r="Z34" s="35"/>
+      <c r="AB34" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="BC34" s="120"/>
-      <c r="BD34" s="120"/>
-      <c r="BE34" s="120"/>
-      <c r="BF34" s="120"/>
-      <c r="BG34" s="120"/>
-      <c r="BH34" s="120"/>
-      <c r="BI34" s="120"/>
-      <c r="BJ34" s="120"/>
-      <c r="BK34" s="120"/>
-      <c r="BL34" s="120"/>
-      <c r="BM34" s="122"/>
+      <c r="AC34" s="34"/>
+      <c r="AD34" s="34"/>
+      <c r="AE34" s="34"/>
+      <c r="AF34" s="34"/>
+      <c r="AG34" s="34"/>
+      <c r="AH34" s="34"/>
+      <c r="AI34" s="34"/>
+      <c r="AJ34" s="34"/>
+      <c r="AK34" s="34"/>
+      <c r="AL34" s="34"/>
+      <c r="AM34" s="35"/>
+      <c r="AO34" s="33" t="s">
+        <v>25</v>
+      </c>
+      <c r="AP34" s="34"/>
+      <c r="AQ34" s="34"/>
+      <c r="AR34" s="34"/>
+      <c r="AS34" s="34"/>
+      <c r="AT34" s="34"/>
+      <c r="AU34" s="34"/>
+      <c r="AV34" s="34"/>
+      <c r="AW34" s="34"/>
+      <c r="AX34" s="34"/>
+      <c r="AY34" s="34"/>
+      <c r="AZ34" s="35"/>
+      <c r="BA34" s="16"/>
+      <c r="BB34" s="33" t="s">
+        <v>25</v>
+      </c>
+      <c r="BC34" s="34"/>
+      <c r="BD34" s="34"/>
+      <c r="BE34" s="34"/>
+      <c r="BF34" s="34"/>
+      <c r="BG34" s="34"/>
+      <c r="BH34" s="34"/>
+      <c r="BI34" s="34"/>
+      <c r="BJ34" s="34"/>
+      <c r="BK34" s="34"/>
+      <c r="BL34" s="34"/>
+      <c r="BM34" s="35"/>
     </row>
     <row r="35" spans="2:65" ht="15" thickTop="1">
       <c r="B35" s="14"/>
@@ -11685,53 +11597,61 @@
       <c r="BM157" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="118">
-    <mergeCell ref="B32:M32"/>
-    <mergeCell ref="AB32:AM32"/>
-    <mergeCell ref="BB32:BM32"/>
-    <mergeCell ref="B33:M33"/>
-    <mergeCell ref="AB33:AM33"/>
-    <mergeCell ref="BB33:BM33"/>
-    <mergeCell ref="AB34:AE34"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="BB34:BE34"/>
-    <mergeCell ref="F34:M34"/>
-    <mergeCell ref="AF34:AM34"/>
-    <mergeCell ref="BF34:BM34"/>
-    <mergeCell ref="AP22:BM23"/>
-    <mergeCell ref="B25:M25"/>
-    <mergeCell ref="AB25:AM25"/>
-    <mergeCell ref="BB25:BM25"/>
-    <mergeCell ref="AN18:AT18"/>
-    <mergeCell ref="AU18:BB18"/>
-    <mergeCell ref="BC18:BM18"/>
-    <mergeCell ref="B20:AO20"/>
-    <mergeCell ref="AP20:BM21"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="I18:U18"/>
-    <mergeCell ref="V18:AG18"/>
-    <mergeCell ref="AH18:AJ18"/>
-    <mergeCell ref="AK18:AM18"/>
-    <mergeCell ref="C21:AN22"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="I17:U17"/>
-    <mergeCell ref="V17:AG17"/>
-    <mergeCell ref="AH17:AJ17"/>
-    <mergeCell ref="AK17:AM17"/>
-    <mergeCell ref="AN17:AT17"/>
-    <mergeCell ref="AU17:BB17"/>
-    <mergeCell ref="BC17:BM17"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="I16:U16"/>
-    <mergeCell ref="V16:AG16"/>
-    <mergeCell ref="AH16:AJ16"/>
-    <mergeCell ref="AK16:AM16"/>
-    <mergeCell ref="AN16:AT16"/>
-    <mergeCell ref="AU16:BB16"/>
-    <mergeCell ref="BC16:BM16"/>
+  <mergeCells count="128">
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="I6:AM6"/>
+    <mergeCell ref="AN6:AQ6"/>
+    <mergeCell ref="AS6:BM6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="I7:AM7"/>
+    <mergeCell ref="AN7:AQ7"/>
+    <mergeCell ref="AS7:BM7"/>
+    <mergeCell ref="G1:AZ2"/>
+    <mergeCell ref="BA1:BF1"/>
+    <mergeCell ref="BH1:BM1"/>
+    <mergeCell ref="BA2:BF2"/>
+    <mergeCell ref="BH2:BM2"/>
+    <mergeCell ref="G3:AZ4"/>
+    <mergeCell ref="BA3:BF3"/>
+    <mergeCell ref="BH3:BM3"/>
+    <mergeCell ref="BA4:BF4"/>
+    <mergeCell ref="BH4:BM4"/>
+    <mergeCell ref="AN9:AT10"/>
+    <mergeCell ref="AU9:BB10"/>
+    <mergeCell ref="BC9:BM10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="I11:U11"/>
+    <mergeCell ref="V11:AG11"/>
+    <mergeCell ref="AH11:AJ11"/>
+    <mergeCell ref="AK11:AM11"/>
+    <mergeCell ref="AN11:AT11"/>
+    <mergeCell ref="B9:C10"/>
+    <mergeCell ref="D9:H10"/>
+    <mergeCell ref="I9:U10"/>
+    <mergeCell ref="V9:AG10"/>
+    <mergeCell ref="AH9:AJ10"/>
+    <mergeCell ref="AK9:AM10"/>
+    <mergeCell ref="AU11:BB11"/>
+    <mergeCell ref="BC11:BM11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="I12:U12"/>
+    <mergeCell ref="V12:AG12"/>
+    <mergeCell ref="AH12:AJ12"/>
+    <mergeCell ref="AK12:AM12"/>
+    <mergeCell ref="AN12:AT12"/>
+    <mergeCell ref="AU12:BB12"/>
+    <mergeCell ref="BC12:BM12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="I13:U13"/>
+    <mergeCell ref="V13:AG13"/>
+    <mergeCell ref="AH13:AJ13"/>
+    <mergeCell ref="AK13:AM13"/>
+    <mergeCell ref="AN13:AT13"/>
+    <mergeCell ref="AU13:BB13"/>
+    <mergeCell ref="BC13:BM13"/>
     <mergeCell ref="AN14:AT14"/>
     <mergeCell ref="AU14:BB14"/>
     <mergeCell ref="BC14:BM14"/>
@@ -11750,63 +11670,65 @@
     <mergeCell ref="AK14:AM14"/>
     <mergeCell ref="AU15:BB15"/>
     <mergeCell ref="BC15:BM15"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="I13:U13"/>
-    <mergeCell ref="V13:AG13"/>
-    <mergeCell ref="AH13:AJ13"/>
-    <mergeCell ref="AK13:AM13"/>
-    <mergeCell ref="AN13:AT13"/>
-    <mergeCell ref="AU13:BB13"/>
-    <mergeCell ref="BC13:BM13"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="I12:U12"/>
-    <mergeCell ref="V12:AG12"/>
-    <mergeCell ref="AH12:AJ12"/>
-    <mergeCell ref="AK12:AM12"/>
-    <mergeCell ref="AN12:AT12"/>
-    <mergeCell ref="AU12:BB12"/>
-    <mergeCell ref="BC12:BM12"/>
-    <mergeCell ref="AN9:AT10"/>
-    <mergeCell ref="AU9:BB10"/>
-    <mergeCell ref="BC9:BM10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="I11:U11"/>
-    <mergeCell ref="V11:AG11"/>
-    <mergeCell ref="AH11:AJ11"/>
-    <mergeCell ref="AK11:AM11"/>
-    <mergeCell ref="AN11:AT11"/>
-    <mergeCell ref="B9:C10"/>
-    <mergeCell ref="D9:H10"/>
-    <mergeCell ref="I9:U10"/>
-    <mergeCell ref="V9:AG10"/>
-    <mergeCell ref="AH9:AJ10"/>
-    <mergeCell ref="AK9:AM10"/>
-    <mergeCell ref="AU11:BB11"/>
-    <mergeCell ref="BC11:BM11"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="I6:AM6"/>
-    <mergeCell ref="AN6:AQ6"/>
-    <mergeCell ref="AS6:BM6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="I7:AM7"/>
-    <mergeCell ref="AN7:AQ7"/>
-    <mergeCell ref="AS7:BM7"/>
-    <mergeCell ref="G1:AZ2"/>
-    <mergeCell ref="BA1:BF1"/>
-    <mergeCell ref="BH1:BM1"/>
-    <mergeCell ref="BA2:BF2"/>
-    <mergeCell ref="BH2:BM2"/>
-    <mergeCell ref="G3:AZ4"/>
-    <mergeCell ref="BA3:BF3"/>
-    <mergeCell ref="BH3:BM3"/>
-    <mergeCell ref="BA4:BF4"/>
-    <mergeCell ref="BH4:BM4"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="I16:U16"/>
+    <mergeCell ref="V16:AG16"/>
+    <mergeCell ref="AH16:AJ16"/>
+    <mergeCell ref="AK16:AM16"/>
+    <mergeCell ref="AN16:AT16"/>
+    <mergeCell ref="AU16:BB16"/>
+    <mergeCell ref="BC16:BM16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="I17:U17"/>
+    <mergeCell ref="V17:AG17"/>
+    <mergeCell ref="AH17:AJ17"/>
+    <mergeCell ref="AK17:AM17"/>
+    <mergeCell ref="AN17:AT17"/>
+    <mergeCell ref="AU17:BB17"/>
+    <mergeCell ref="BC17:BM17"/>
+    <mergeCell ref="AP22:BM23"/>
+    <mergeCell ref="B25:M25"/>
+    <mergeCell ref="AB25:AM25"/>
+    <mergeCell ref="BB25:BM25"/>
+    <mergeCell ref="AN18:AT18"/>
+    <mergeCell ref="AU18:BB18"/>
+    <mergeCell ref="BC18:BM18"/>
+    <mergeCell ref="B20:AO20"/>
+    <mergeCell ref="AP20:BM21"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="I18:U18"/>
+    <mergeCell ref="V18:AG18"/>
+    <mergeCell ref="AH18:AJ18"/>
+    <mergeCell ref="AK18:AM18"/>
+    <mergeCell ref="C21:AN22"/>
+    <mergeCell ref="O25:Z25"/>
+    <mergeCell ref="AO25:AZ25"/>
+    <mergeCell ref="B32:M32"/>
+    <mergeCell ref="AB32:AM32"/>
+    <mergeCell ref="BB32:BM32"/>
+    <mergeCell ref="B33:M33"/>
+    <mergeCell ref="AB33:AM33"/>
+    <mergeCell ref="BB33:BM33"/>
+    <mergeCell ref="AB34:AE34"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="BB34:BE34"/>
+    <mergeCell ref="F34:M34"/>
+    <mergeCell ref="AF34:AM34"/>
+    <mergeCell ref="BF34:BM34"/>
+    <mergeCell ref="O32:Z32"/>
+    <mergeCell ref="O33:Z33"/>
+    <mergeCell ref="O34:R34"/>
+    <mergeCell ref="S34:Z34"/>
+    <mergeCell ref="AO32:AZ32"/>
+    <mergeCell ref="AO33:AZ33"/>
+    <mergeCell ref="AO34:AR34"/>
+    <mergeCell ref="AS34:AZ34"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="78" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="77" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <rowBreaks count="4" manualBreakCount="4">
     <brk id="51" max="51" man="1"/>
     <brk id="81" max="51" man="1"/>

</xml_diff>